<commit_message>
Updated plot with ratio percentages and user input for affected wrist
</commit_message>
<xml_diff>
--- a/outputs/results/subject_energy/orientation_energy.xlsx
+++ b/outputs/results/subject_energy/orientation_energy.xlsx
@@ -496,11 +496,11 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>369.7999877929688</v>
+        <v>36980</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>369.7999877929688</v>
+        <v>36980</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" s="1" t="n">
@@ -527,16 +527,16 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>282.1000061035156</v>
+        <v>28210</v>
       </c>
       <c r="H3" t="n">
-        <v>427.8999938964844</v>
+        <v>42790</v>
       </c>
       <c r="I3" t="n">
-        <v>710</v>
+        <v>71000</v>
       </c>
       <c r="J3" t="n">
-        <v>0.6592662073553569</v>
+        <v>0.6592661836877776</v>
       </c>
       <c r="K3" s="1" t="n">
         <v>46100.625</v>
@@ -561,10 +561,10 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>427.8999938964844</v>
+        <v>42790</v>
       </c>
       <c r="I4" t="n">
-        <v>427.8999938964844</v>
+        <v>42790</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" s="1" t="n">
@@ -591,16 +591,16 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>236.5</v>
+        <v>23650</v>
       </c>
       <c r="H5" t="n">
-        <v>427.8999938964844</v>
+        <v>42790</v>
       </c>
       <c r="I5" t="n">
-        <v>664.3999938964844</v>
+        <v>66440</v>
       </c>
       <c r="J5" t="n">
-        <v>0.5526992366754111</v>
+        <v>0.5526992287917738</v>
       </c>
       <c r="K5" s="1" t="n">
         <v>46100.625</v>
@@ -625,10 +625,10 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>402.1000061035156</v>
+        <v>40210</v>
       </c>
       <c r="I6" t="n">
-        <v>402.1000061035156</v>
+        <v>40210</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" s="1" t="n">
@@ -655,16 +655,16 @@
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>212.8000030517578</v>
+        <v>21280</v>
       </c>
       <c r="H7" t="n">
-        <v>402.1000061035156</v>
+        <v>40210</v>
       </c>
       <c r="I7" t="n">
-        <v>614.9000091552734</v>
+        <v>61490</v>
       </c>
       <c r="J7" t="n">
-        <v>0.5292215862264252</v>
+        <v>0.5292215866699826</v>
       </c>
       <c r="K7" s="1" t="n">
         <v>46100.625</v>
@@ -689,10 +689,10 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>329.1000061035156</v>
+        <v>32910</v>
       </c>
       <c r="I8" t="n">
-        <v>329.1000061035156</v>
+        <v>32910</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" s="1" t="n">
@@ -719,16 +719,16 @@
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>187.5</v>
+        <v>18750</v>
       </c>
       <c r="H9" t="n">
-        <v>329.1000061035156</v>
+        <v>32910</v>
       </c>
       <c r="I9" t="n">
-        <v>516.6000061035156</v>
+        <v>51660</v>
       </c>
       <c r="J9" t="n">
-        <v>0.5697356320954411</v>
+        <v>0.5697356426618049</v>
       </c>
       <c r="K9" s="1" t="n">
         <v>46100.625</v>
@@ -753,10 +753,10 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>270.2000122070312</v>
+        <v>27020</v>
       </c>
       <c r="I10" t="n">
-        <v>270.2000122070312</v>
+        <v>27020</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" s="1" t="n">
@@ -783,16 +783,16 @@
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>168.1000061035156</v>
+        <v>16810</v>
       </c>
       <c r="H11" t="n">
-        <v>270.2000122070312</v>
+        <v>27020</v>
       </c>
       <c r="I11" t="n">
-        <v>438.3000183105469</v>
+        <v>43830</v>
       </c>
       <c r="J11" t="n">
-        <v>0.6221317487384675</v>
+        <v>0.6221317542561066</v>
       </c>
       <c r="K11" s="1" t="n">
         <v>46100.625</v>
@@ -817,10 +817,10 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>247.8000030517578</v>
+        <v>24780</v>
       </c>
       <c r="I12" t="n">
-        <v>247.8000030517578</v>
+        <v>24780</v>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" s="1" t="n">
@@ -847,16 +847,16 @@
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>164.5</v>
+        <v>16450</v>
       </c>
       <c r="H13" t="n">
-        <v>247.8000030517578</v>
+        <v>24780</v>
       </c>
       <c r="I13" t="n">
-        <v>412.3000030517578</v>
+        <v>41230</v>
       </c>
       <c r="J13" t="n">
-        <v>0.6638417997341227</v>
+        <v>0.6638418079096046</v>
       </c>
       <c r="K13" s="1" t="n">
         <v>46100.625</v>
@@ -881,10 +881,10 @@
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>231.1000061035156</v>
+        <v>23110</v>
       </c>
       <c r="I14" t="n">
-        <v>231.1000061035156</v>
+        <v>23110</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" s="1" t="n">
@@ -911,16 +911,16 @@
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>173.1000061035156</v>
+        <v>17310</v>
       </c>
       <c r="H15" t="n">
-        <v>231.1000061035156</v>
+        <v>23110</v>
       </c>
       <c r="I15" t="n">
-        <v>404.2000122070312</v>
+        <v>40420</v>
       </c>
       <c r="J15" t="n">
-        <v>0.7490264021281752</v>
+        <v>0.7490263954997837</v>
       </c>
       <c r="K15" s="1" t="n">
         <v>46100.625</v>
@@ -945,10 +945,10 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>205.5</v>
+        <v>20550</v>
       </c>
       <c r="I16" t="n">
-        <v>205.5</v>
+        <v>20550</v>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" s="1" t="n">
@@ -975,16 +975,16 @@
         <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>177.1999969482422</v>
+        <v>17720</v>
       </c>
       <c r="H17" t="n">
-        <v>205.5</v>
+        <v>20550</v>
       </c>
       <c r="I17" t="n">
-        <v>382.6999969482422</v>
+        <v>38270</v>
       </c>
       <c r="J17" t="n">
-        <v>0.862287089772468</v>
+        <v>0.8622871046228711</v>
       </c>
       <c r="K17" s="1" t="n">
         <v>46100.625</v>
@@ -1009,10 +1009,10 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>196.1000061035156</v>
+        <v>19610</v>
       </c>
       <c r="I18" t="n">
-        <v>196.1000061035156</v>
+        <v>19610</v>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" s="1" t="n">
@@ -1039,16 +1039,16 @@
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>174.6000061035156</v>
+        <v>17460</v>
       </c>
       <c r="H19" t="n">
-        <v>196.1000061035156</v>
+        <v>19610</v>
       </c>
       <c r="I19" t="n">
-        <v>370.7000122070312</v>
+        <v>37070</v>
       </c>
       <c r="J19" t="n">
-        <v>0.8903620635858075</v>
+        <v>0.8903620601733809</v>
       </c>
       <c r="K19" s="1" t="n">
         <v>46100.625</v>
@@ -1073,10 +1073,10 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>198.1999969482422</v>
+        <v>19820</v>
       </c>
       <c r="I20" t="n">
-        <v>198.1999969482422</v>
+        <v>19820</v>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" s="1" t="n">
@@ -1103,16 +1103,16 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>171.5</v>
+        <v>17150</v>
       </c>
       <c r="H21" t="n">
-        <v>198.1999969482422</v>
+        <v>19820</v>
       </c>
       <c r="I21" t="n">
-        <v>369.6999969482422</v>
+        <v>36970</v>
       </c>
       <c r="J21" t="n">
-        <v>0.8652876016178012</v>
+        <v>0.8652875882946519</v>
       </c>
       <c r="K21" s="1" t="n">
         <v>46100.625</v>
@@ -1137,10 +1137,10 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>197</v>
+        <v>19700</v>
       </c>
       <c r="I22" t="n">
-        <v>197</v>
+        <v>19700</v>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" s="1" t="n">
@@ -1167,16 +1167,16 @@
         <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>177.8000030517578</v>
+        <v>17780</v>
       </c>
       <c r="H23" t="n">
-        <v>197</v>
+        <v>19700</v>
       </c>
       <c r="I23" t="n">
-        <v>374.8000030517578</v>
+        <v>37480</v>
       </c>
       <c r="J23" t="n">
-        <v>0.9025380865571463</v>
+        <v>0.9025380710659898</v>
       </c>
       <c r="K23" s="1" t="n">
         <v>46100.625</v>
@@ -1201,10 +1201,10 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>185.5</v>
+        <v>18550</v>
       </c>
       <c r="I24" t="n">
-        <v>185.5</v>
+        <v>18550</v>
       </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" s="1" t="n">
@@ -1231,16 +1231,16 @@
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>185.1999969482422</v>
+        <v>18520</v>
       </c>
       <c r="H25" t="n">
-        <v>185.5</v>
+        <v>18550</v>
       </c>
       <c r="I25" t="n">
-        <v>370.6999969482422</v>
+        <v>37070</v>
       </c>
       <c r="J25" t="n">
-        <v>0.998382732874621</v>
+        <v>0.9983827493261456</v>
       </c>
       <c r="K25" s="1" t="n">
         <v>46100.625</v>
@@ -1265,10 +1265,10 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>176.1000061035156</v>
+        <v>17610</v>
       </c>
       <c r="I26" t="n">
-        <v>176.1000061035156</v>
+        <v>17610</v>
       </c>
       <c r="J26" t="inlineStr"/>
       <c r="K26" s="1" t="n">
@@ -1295,16 +1295,16 @@
         <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>184</v>
+        <v>18400</v>
       </c>
       <c r="H27" t="n">
-        <v>176.1000061035156</v>
+        <v>17610</v>
       </c>
       <c r="I27" t="n">
-        <v>360.1000061035156</v>
+        <v>36010</v>
       </c>
       <c r="J27" t="n">
-        <v>1.044860838288902</v>
+        <v>1.044860874503123</v>
       </c>
       <c r="K27" s="1" t="n">
         <v>46100.625</v>
@@ -1329,10 +1329,10 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>173.3999938964844</v>
+        <v>17340</v>
       </c>
       <c r="I28" t="n">
-        <v>173.3999938964844</v>
+        <v>17340</v>
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" s="1" t="n">
@@ -1359,16 +1359,16 @@
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>185.6999969482422</v>
+        <v>18570</v>
       </c>
       <c r="H29" t="n">
-        <v>173.3999938964844</v>
+        <v>17340</v>
       </c>
       <c r="I29" t="n">
-        <v>359.0999908447266</v>
+        <v>35910</v>
       </c>
       <c r="J29" t="n">
-        <v>1.070934276151709</v>
+        <v>1.070934256055363</v>
       </c>
       <c r="K29" s="1" t="n">
         <v>46100.625</v>
@@ -1393,10 +1393,10 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>170.6999969482422</v>
+        <v>17070</v>
       </c>
       <c r="I30" t="n">
-        <v>170.6999969482422</v>
+        <v>17070</v>
       </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" s="1" t="n">
@@ -1423,16 +1423,16 @@
         <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>182.6999969482422</v>
+        <v>18270</v>
       </c>
       <c r="H31" t="n">
-        <v>170.6999969482422</v>
+        <v>17070</v>
       </c>
       <c r="I31" t="n">
-        <v>353.3999938964844</v>
+        <v>35340</v>
       </c>
       <c r="J31" t="n">
-        <v>1.070298771028324</v>
+        <v>1.070298769771529</v>
       </c>
       <c r="K31" s="1" t="n">
         <v>46100.625</v>
@@ -1457,10 +1457,10 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>169.1999969482422</v>
+        <v>16920</v>
       </c>
       <c r="I32" t="n">
-        <v>169.1999969482422</v>
+        <v>16920</v>
       </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" s="1" t="n">
@@ -1487,16 +1487,16 @@
         <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>173.8999938964844</v>
+        <v>17390</v>
       </c>
       <c r="H33" t="n">
-        <v>169.1999969482422</v>
+        <v>16920</v>
       </c>
       <c r="I33" t="n">
-        <v>343.0999908447266</v>
+        <v>34310</v>
       </c>
       <c r="J33" t="n">
-        <v>1.027777760242395</v>
+        <v>1.027777777777778</v>
       </c>
       <c r="K33" s="1" t="n">
         <v>46100.625</v>
@@ -1521,10 +1521,10 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>175.6000061035156</v>
+        <v>17560</v>
       </c>
       <c r="I34" t="n">
-        <v>175.6000061035156</v>
+        <v>17560</v>
       </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" s="1" t="n">
@@ -1551,16 +1551,16 @@
         <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>174.1000061035156</v>
+        <v>17410</v>
       </c>
       <c r="H35" t="n">
-        <v>175.6000061035156</v>
+        <v>17560</v>
       </c>
       <c r="I35" t="n">
-        <v>349.7000122070312</v>
+        <v>34970</v>
       </c>
       <c r="J35" t="n">
-        <v>0.9914578590668399</v>
+        <v>0.9914578587699316</v>
       </c>
       <c r="K35" s="1" t="n">
         <v>46100.625</v>
@@ -1585,10 +1585,10 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>186.5</v>
+        <v>18650</v>
       </c>
       <c r="I36" t="n">
-        <v>186.5</v>
+        <v>18650</v>
       </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" s="1" t="n">
@@ -1615,16 +1615,16 @@
         <v>1</v>
       </c>
       <c r="G37" t="n">
-        <v>176.3999938964844</v>
+        <v>17640</v>
       </c>
       <c r="H37" t="n">
-        <v>186.5</v>
+        <v>18650</v>
       </c>
       <c r="I37" t="n">
-        <v>362.8999938964844</v>
+        <v>36290</v>
       </c>
       <c r="J37" t="n">
-        <v>0.9458444712948224</v>
+        <v>0.9458445040214477</v>
       </c>
       <c r="K37" s="1" t="n">
         <v>46100.625</v>
@@ -1649,10 +1649,10 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>185</v>
+        <v>18500</v>
       </c>
       <c r="I38" t="n">
-        <v>185</v>
+        <v>18500</v>
       </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" s="1" t="n">
@@ -1679,16 +1679,16 @@
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>178.6999969482422</v>
+        <v>17870</v>
       </c>
       <c r="H39" t="n">
-        <v>185</v>
+        <v>18500</v>
       </c>
       <c r="I39" t="n">
-        <v>363.6999969482422</v>
+        <v>36370</v>
       </c>
       <c r="J39" t="n">
-        <v>0.9659459294499577</v>
+        <v>0.965945945945946</v>
       </c>
       <c r="K39" s="1" t="n">
         <v>46100.625</v>
@@ -1713,10 +1713,10 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>172.6999969482422</v>
+        <v>17270</v>
       </c>
       <c r="I40" t="n">
-        <v>172.6999969482422</v>
+        <v>17270</v>
       </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" s="1" t="n">
@@ -1743,16 +1743,16 @@
         <v>1</v>
       </c>
       <c r="G41" t="n">
-        <v>180.1000061035156</v>
+        <v>18010</v>
       </c>
       <c r="H41" t="n">
-        <v>172.6999969482422</v>
+        <v>17270</v>
       </c>
       <c r="I41" t="n">
-        <v>352.8000030517578</v>
+        <v>35280</v>
       </c>
       <c r="J41" t="n">
-        <v>1.042848924644111</v>
+        <v>1.042848870874349</v>
       </c>
       <c r="K41" s="1" t="n">
         <v>46100.625</v>
@@ -1777,10 +1777,10 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>165.8999938964844</v>
+        <v>16590</v>
       </c>
       <c r="I42" t="n">
-        <v>165.8999938964844</v>
+        <v>16590</v>
       </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" s="1" t="n">
@@ -1807,16 +1807,16 @@
         <v>1</v>
       </c>
       <c r="G43" t="n">
-        <v>175.6999969482422</v>
+        <v>17570</v>
       </c>
       <c r="H43" t="n">
-        <v>165.8999938964844</v>
+        <v>16590</v>
       </c>
       <c r="I43" t="n">
-        <v>341.5999908447266</v>
+        <v>34160</v>
       </c>
       <c r="J43" t="n">
-        <v>1.05907175052624</v>
+        <v>1.059071729957806</v>
       </c>
       <c r="K43" s="1" t="n">
         <v>46100.625</v>
@@ -1841,10 +1841,10 @@
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>167.1999969482422</v>
+        <v>16720</v>
       </c>
       <c r="I44" t="n">
-        <v>167.1999969482422</v>
+        <v>16720</v>
       </c>
       <c r="J44" t="inlineStr"/>
       <c r="K44" s="1" t="n">
@@ -1871,16 +1871,16 @@
         <v>1</v>
       </c>
       <c r="G45" t="n">
-        <v>173</v>
+        <v>17300</v>
       </c>
       <c r="H45" t="n">
-        <v>167.1999969482422</v>
+        <v>16720</v>
       </c>
       <c r="I45" t="n">
-        <v>340.1999969482422</v>
+        <v>34020</v>
       </c>
       <c r="J45" t="n">
-        <v>1.0346890141006</v>
+        <v>1.034688995215311</v>
       </c>
       <c r="K45" s="1" t="n">
         <v>46100.625</v>
@@ -1905,10 +1905,10 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>164.1999969482422</v>
+        <v>16420</v>
       </c>
       <c r="I46" t="n">
-        <v>164.1999969482422</v>
+        <v>16420</v>
       </c>
       <c r="J46" t="inlineStr"/>
       <c r="K46" s="1" t="n">
@@ -1935,16 +1935,16 @@
         <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>172.6999969482422</v>
+        <v>17270</v>
       </c>
       <c r="H47" t="n">
-        <v>164.1999969482422</v>
+        <v>16420</v>
       </c>
       <c r="I47" t="n">
-        <v>336.8999938964844</v>
+        <v>33690</v>
       </c>
       <c r="J47" t="n">
-        <v>1.05176613981716</v>
+        <v>1.051766138855055</v>
       </c>
       <c r="K47" s="1" t="n">
         <v>46100.625</v>
@@ -1969,10 +1969,10 @@
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>155.8999938964844</v>
+        <v>15590</v>
       </c>
       <c r="I48" t="n">
-        <v>155.8999938964844</v>
+        <v>15590</v>
       </c>
       <c r="J48" t="inlineStr"/>
       <c r="K48" s="1" t="n">
@@ -1999,16 +1999,16 @@
         <v>1</v>
       </c>
       <c r="G49" t="n">
-        <v>169.1000061035156</v>
+        <v>16910</v>
       </c>
       <c r="H49" t="n">
-        <v>155.8999938964844</v>
+        <v>15590</v>
       </c>
       <c r="I49" t="n">
-        <v>325</v>
+        <v>32500</v>
       </c>
       <c r="J49" t="n">
-        <v>1.084669741653716</v>
+        <v>1.084669660038486</v>
       </c>
       <c r="K49" s="1" t="n">
         <v>46100.625</v>
@@ -2033,10 +2033,10 @@
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>151.6999969482422</v>
+        <v>15170</v>
       </c>
       <c r="I50" t="n">
-        <v>151.6999969482422</v>
+        <v>15170</v>
       </c>
       <c r="J50" t="inlineStr"/>
       <c r="K50" s="1" t="n">
@@ -2063,16 +2063,16 @@
         <v>1</v>
       </c>
       <c r="G51" t="n">
-        <v>166.6999969482422</v>
+        <v>16670</v>
       </c>
       <c r="H51" t="n">
-        <v>151.6999969482422</v>
+        <v>15170</v>
       </c>
       <c r="I51" t="n">
-        <v>318.3999938964844</v>
+        <v>31840</v>
       </c>
       <c r="J51" t="n">
-        <v>1.098879369161212</v>
+        <v>1.09887936717205</v>
       </c>
       <c r="K51" s="1" t="n">
         <v>46100.625</v>
@@ -2097,10 +2097,10 @@
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>152.1999969482422</v>
+        <v>15220</v>
       </c>
       <c r="I52" t="n">
-        <v>152.1999969482422</v>
+        <v>15220</v>
       </c>
       <c r="J52" t="inlineStr"/>
       <c r="K52" s="1" t="n">
@@ -2127,16 +2127,16 @@
         <v>1</v>
       </c>
       <c r="G53" t="n">
-        <v>167.3999938964844</v>
+        <v>16740</v>
       </c>
       <c r="H53" t="n">
-        <v>152.1999969482422</v>
+        <v>15220</v>
       </c>
       <c r="I53" t="n">
-        <v>319.5999908447266</v>
+        <v>31960</v>
       </c>
       <c r="J53" t="n">
-        <v>1.099868575906813</v>
+        <v>1.099868593955322</v>
       </c>
       <c r="K53" s="1" t="n">
         <v>46100.625</v>
@@ -2161,10 +2161,10 @@
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>157.1000061035156</v>
+        <v>15710</v>
       </c>
       <c r="I54" t="n">
-        <v>157.1000061035156</v>
+        <v>15710</v>
       </c>
       <c r="J54" t="inlineStr"/>
       <c r="K54" s="1" t="n">
@@ -2191,16 +2191,16 @@
         <v>1</v>
       </c>
       <c r="G55" t="n">
-        <v>166.3000030517578</v>
+        <v>16630</v>
       </c>
       <c r="H55" t="n">
-        <v>157.1000061035156</v>
+        <v>15710</v>
       </c>
       <c r="I55" t="n">
-        <v>323.4000091552734</v>
+        <v>32340</v>
       </c>
       <c r="J55" t="n">
-        <v>1.058561404142659</v>
+        <v>1.058561425843412</v>
       </c>
       <c r="K55" s="1" t="n">
         <v>46100.625</v>
@@ -2225,10 +2225,10 @@
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>159</v>
+        <v>15900</v>
       </c>
       <c r="I56" t="n">
-        <v>159</v>
+        <v>15900</v>
       </c>
       <c r="J56" t="inlineStr"/>
       <c r="K56" s="1" t="n">
@@ -2255,16 +2255,16 @@
         <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>168.6999969482422</v>
+        <v>16870</v>
       </c>
       <c r="H57" t="n">
-        <v>159</v>
+        <v>15900</v>
       </c>
       <c r="I57" t="n">
-        <v>327.6999969482422</v>
+        <v>32770</v>
       </c>
       <c r="J57" t="n">
-        <v>1.061006270114731</v>
+        <v>1.061006289308176</v>
       </c>
       <c r="K57" s="1" t="n">
         <v>46100.625</v>
@@ -2289,10 +2289,10 @@
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>164</v>
+        <v>16400</v>
       </c>
       <c r="I58" t="n">
-        <v>164</v>
+        <v>16400</v>
       </c>
       <c r="J58" t="inlineStr"/>
       <c r="K58" s="1" t="n">
@@ -2319,16 +2319,16 @@
         <v>1</v>
       </c>
       <c r="G59" t="n">
-        <v>181.6999969482422</v>
+        <v>18170</v>
       </c>
       <c r="H59" t="n">
-        <v>164</v>
+        <v>16400</v>
       </c>
       <c r="I59" t="n">
-        <v>345.6999969482422</v>
+        <v>34570</v>
       </c>
       <c r="J59" t="n">
-        <v>1.107926810660013</v>
+        <v>1.107926829268293</v>
       </c>
       <c r="K59" s="1" t="n">
         <v>46100.625</v>
@@ -2353,10 +2353,10 @@
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>180.1000061035156</v>
+        <v>18010</v>
       </c>
       <c r="I60" t="n">
-        <v>180.1000061035156</v>
+        <v>18010</v>
       </c>
       <c r="J60" t="inlineStr"/>
       <c r="K60" s="1" t="n">
@@ -2383,16 +2383,16 @@
         <v>1</v>
       </c>
       <c r="G61" t="n">
-        <v>200.1000061035156</v>
+        <v>20010</v>
       </c>
       <c r="H61" t="n">
-        <v>180.1000061035156</v>
+        <v>18010</v>
       </c>
       <c r="I61" t="n">
-        <v>380.2000122070312</v>
+        <v>38020</v>
       </c>
       <c r="J61" t="n">
-        <v>1.111049413227141</v>
+        <v>1.111049416990561</v>
       </c>
       <c r="K61" s="1" t="n">
         <v>46100.625</v>
@@ -2417,10 +2417,10 @@
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="n">
-        <v>184.1000061035156</v>
+        <v>18410</v>
       </c>
       <c r="I62" t="n">
-        <v>184.1000061035156</v>
+        <v>18410</v>
       </c>
       <c r="J62" t="inlineStr"/>
       <c r="K62" s="1" t="n">
@@ -2447,16 +2447,16 @@
         <v>1</v>
       </c>
       <c r="G63" t="n">
-        <v>178</v>
+        <v>17800</v>
       </c>
       <c r="H63" t="n">
-        <v>184.1000061035156</v>
+        <v>18410</v>
       </c>
       <c r="I63" t="n">
-        <v>362.1000061035156</v>
+        <v>36210</v>
       </c>
       <c r="J63" t="n">
-        <v>0.9668658017312302</v>
+        <v>0.9668658337859859</v>
       </c>
       <c r="K63" s="1" t="n">
         <v>46100.625</v>
@@ -2481,10 +2481,10 @@
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="n">
-        <v>163.6999969482422</v>
+        <v>16370</v>
       </c>
       <c r="I64" t="n">
-        <v>163.6999969482422</v>
+        <v>16370</v>
       </c>
       <c r="J64" t="inlineStr"/>
       <c r="K64" s="1" t="n">
@@ -2511,16 +2511,16 @@
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>227</v>
+        <v>22700</v>
       </c>
       <c r="H65" t="n">
-        <v>163.6999969482422</v>
+        <v>16370</v>
       </c>
       <c r="I65" t="n">
-        <v>390.6999969482422</v>
+        <v>39070</v>
       </c>
       <c r="J65" t="n">
-        <v>1.386682982479051</v>
+        <v>1.386682956627978</v>
       </c>
       <c r="K65" s="1" t="n">
         <v>46100.625</v>
@@ -2545,10 +2545,10 @@
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="n">
-        <v>159.8000030517578</v>
+        <v>15980</v>
       </c>
       <c r="I66" t="n">
-        <v>159.8000030517578</v>
+        <v>15980</v>
       </c>
       <c r="J66" t="inlineStr"/>
       <c r="K66" s="1" t="n">
@@ -2575,16 +2575,16 @@
         <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>312.6000061035156</v>
+        <v>31260</v>
       </c>
       <c r="H67" t="n">
-        <v>159.8000030517578</v>
+        <v>15980</v>
       </c>
       <c r="I67" t="n">
-        <v>472.4000091552734</v>
+        <v>47240</v>
       </c>
       <c r="J67" t="n">
-        <v>1.956195244891624</v>
+        <v>1.956195244055069</v>
       </c>
       <c r="K67" s="1" t="n">
         <v>46100.625</v>
@@ -2609,10 +2609,10 @@
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
-        <v>173.8999938964844</v>
+        <v>17390</v>
       </c>
       <c r="I68" t="n">
-        <v>173.8999938964844</v>
+        <v>17390</v>
       </c>
       <c r="J68" t="inlineStr"/>
       <c r="K68" s="1" t="n">
@@ -2639,16 +2639,16 @@
         <v>0</v>
       </c>
       <c r="G69" t="n">
-        <v>367.2999877929688</v>
+        <v>36730</v>
       </c>
       <c r="H69" t="n">
-        <v>173.8999938964844</v>
+        <v>17390</v>
       </c>
       <c r="I69" t="n">
-        <v>541.1999816894531</v>
+        <v>54120</v>
       </c>
       <c r="J69" t="n">
-        <v>2.112133413941392</v>
+        <v>2.11213341000575</v>
       </c>
       <c r="K69" s="1" t="n">
         <v>46100.625</v>
@@ -2673,10 +2673,10 @@
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>199.3000030517578</v>
+        <v>19930</v>
       </c>
       <c r="I70" t="n">
-        <v>199.3000030517578</v>
+        <v>19930</v>
       </c>
       <c r="J70" t="inlineStr"/>
       <c r="K70" s="1" t="n">
@@ -2703,16 +2703,16 @@
         <v>0</v>
       </c>
       <c r="G71" t="n">
-        <v>400.7999877929688</v>
+        <v>40080</v>
       </c>
       <c r="H71" t="n">
-        <v>199.3000030517578</v>
+        <v>19930</v>
       </c>
       <c r="I71" t="n">
-        <v>600.0999908447266</v>
+        <v>60010</v>
       </c>
       <c r="J71" t="n">
-        <v>2.011038543179961</v>
+        <v>2.011038635223282</v>
       </c>
       <c r="K71" s="1" t="n">
         <v>46100.625</v>
@@ -2737,10 +2737,10 @@
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="n">
-        <v>270.3999938964844</v>
+        <v>27040</v>
       </c>
       <c r="I72" t="n">
-        <v>270.3999938964844</v>
+        <v>27040</v>
       </c>
       <c r="J72" t="inlineStr"/>
       <c r="K72" s="1" t="n">
@@ -2767,16 +2767,16 @@
         <v>1</v>
       </c>
       <c r="G73" t="n">
-        <v>419.8999938964844</v>
+        <v>41990</v>
       </c>
       <c r="H73" t="n">
-        <v>270.3999938964844</v>
+        <v>27040</v>
       </c>
       <c r="I73" t="n">
-        <v>690.2999877929688</v>
+        <v>69030</v>
       </c>
       <c r="J73" t="n">
-        <v>1.552884627864423</v>
+        <v>1.552884615384615</v>
       </c>
       <c r="K73" s="1" t="n">
         <v>46100.625</v>
@@ -2801,10 +2801,10 @@
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="n">
-        <v>342.2000122070312</v>
+        <v>34220</v>
       </c>
       <c r="I74" t="n">
-        <v>342.2000122070312</v>
+        <v>34220</v>
       </c>
       <c r="J74" t="inlineStr"/>
       <c r="K74" s="1" t="n">
@@ -2831,16 +2831,16 @@
         <v>1</v>
       </c>
       <c r="G75" t="n">
-        <v>387.6000061035156</v>
+        <v>38760</v>
       </c>
       <c r="H75" t="n">
-        <v>342.2000122070312</v>
+        <v>34220</v>
       </c>
       <c r="I75" t="n">
-        <v>729.8000183105469</v>
+        <v>72980</v>
       </c>
       <c r="J75" t="n">
-        <v>1.132670930090492</v>
+        <v>1.132670952659264</v>
       </c>
       <c r="K75" s="1" t="n">
         <v>46100.625</v>
@@ -2865,10 +2865,10 @@
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>321.5</v>
+        <v>32150</v>
       </c>
       <c r="I76" t="n">
-        <v>321.5</v>
+        <v>32150</v>
       </c>
       <c r="J76" t="inlineStr"/>
       <c r="K76" s="1" t="n">
@@ -2895,16 +2895,16 @@
         <v>1</v>
       </c>
       <c r="G77" t="n">
-        <v>308.7999877929688</v>
+        <v>30880</v>
       </c>
       <c r="H77" t="n">
-        <v>321.5</v>
+        <v>32150</v>
       </c>
       <c r="I77" t="n">
-        <v>630.2999877929688</v>
+        <v>63030</v>
       </c>
       <c r="J77" t="n">
-        <v>0.960497629216077</v>
+        <v>0.96049766718507</v>
       </c>
       <c r="K77" s="1" t="n">
         <v>46100.625</v>
@@ -2929,10 +2929,10 @@
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>247.3999938964844</v>
+        <v>24740</v>
       </c>
       <c r="I78" t="n">
-        <v>247.3999938964844</v>
+        <v>24740</v>
       </c>
       <c r="J78" t="inlineStr"/>
       <c r="K78" s="1" t="n">
@@ -2959,13 +2959,13 @@
         <v>1</v>
       </c>
       <c r="G79" t="n">
-        <v>247.3999938964844</v>
+        <v>24740</v>
       </c>
       <c r="H79" t="n">
-        <v>247.3999938964844</v>
+        <v>24740</v>
       </c>
       <c r="I79" t="n">
-        <v>494.7999877929688</v>
+        <v>49480</v>
       </c>
       <c r="J79" t="n">
         <v>1</v>
@@ -2993,10 +2993,10 @@
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>217.8000030517578</v>
+        <v>21780</v>
       </c>
       <c r="I80" t="n">
-        <v>217.8000030517578</v>
+        <v>21780</v>
       </c>
       <c r="J80" t="inlineStr"/>
       <c r="K80" s="1" t="n">
@@ -3023,16 +3023,16 @@
         <v>1</v>
       </c>
       <c r="G81" t="n">
-        <v>240.3999938964844</v>
+        <v>24040</v>
       </c>
       <c r="H81" t="n">
-        <v>217.8000030517578</v>
+        <v>21780</v>
       </c>
       <c r="I81" t="n">
-        <v>458.1999969482422</v>
+        <v>45820</v>
       </c>
       <c r="J81" t="n">
-        <v>1.103764878457582</v>
+        <v>1.10376492194674</v>
       </c>
       <c r="K81" s="1" t="n">
         <v>46100.625</v>
@@ -3057,10 +3057,10 @@
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>248.8000030517578</v>
+        <v>24880</v>
       </c>
       <c r="I82" t="n">
-        <v>248.8000030517578</v>
+        <v>24880</v>
       </c>
       <c r="J82" t="inlineStr"/>
       <c r="K82" s="1" t="n">
@@ -3087,16 +3087,16 @@
         <v>1</v>
       </c>
       <c r="G83" t="n">
-        <v>284.2999877929688</v>
+        <v>28430</v>
       </c>
       <c r="H83" t="n">
-        <v>248.8000030517578</v>
+        <v>24880</v>
       </c>
       <c r="I83" t="n">
-        <v>533.0999908447266</v>
+        <v>53310</v>
       </c>
       <c r="J83" t="n">
-        <v>1.14268482438011</v>
+        <v>1.142684887459807</v>
       </c>
       <c r="K83" s="1" t="n">
         <v>46100.625</v>
@@ -3121,10 +3121,10 @@
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>288.7999877929688</v>
+        <v>28880</v>
       </c>
       <c r="I84" t="n">
-        <v>288.7999877929688</v>
+        <v>28880</v>
       </c>
       <c r="J84" t="inlineStr"/>
       <c r="K84" s="1" t="n">
@@ -3151,16 +3151,16 @@
         <v>1</v>
       </c>
       <c r="G85" t="n">
-        <v>355.8999938964844</v>
+        <v>35590</v>
       </c>
       <c r="H85" t="n">
-        <v>288.7999877929688</v>
+        <v>28880</v>
       </c>
       <c r="I85" t="n">
-        <v>644.6999816894531</v>
+        <v>64470</v>
       </c>
       <c r="J85" t="n">
-        <v>1.232340751176269</v>
+        <v>1.232340720221607</v>
       </c>
       <c r="K85" s="1" t="n">
         <v>46100.625</v>
@@ -3185,10 +3185,10 @@
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>323.5</v>
+        <v>32350</v>
       </c>
       <c r="I86" t="n">
-        <v>323.5</v>
+        <v>32350</v>
       </c>
       <c r="J86" t="inlineStr"/>
       <c r="K86" s="1" t="n">
@@ -3215,16 +3215,16 @@
         <v>1</v>
       </c>
       <c r="G87" t="n">
-        <v>503.6000061035156</v>
+        <v>50360</v>
       </c>
       <c r="H87" t="n">
-        <v>323.5</v>
+        <v>32350</v>
       </c>
       <c r="I87" t="n">
-        <v>827.1000061035156</v>
+        <v>82710</v>
       </c>
       <c r="J87" t="n">
-        <v>1.556723357352444</v>
+        <v>1.556723338485317</v>
       </c>
       <c r="K87" s="1" t="n">
         <v>46100.625</v>
@@ -3249,10 +3249,10 @@
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>352.6000061035156</v>
+        <v>35260</v>
       </c>
       <c r="I88" t="n">
-        <v>352.6000061035156</v>
+        <v>35260</v>
       </c>
       <c r="J88" t="inlineStr"/>
       <c r="K88" s="1" t="n">
@@ -3279,16 +3279,16 @@
         <v>0</v>
       </c>
       <c r="G89" t="n">
-        <v>744.9000244140625</v>
+        <v>74490</v>
       </c>
       <c r="H89" t="n">
-        <v>352.6000061035156</v>
+        <v>35260</v>
       </c>
       <c r="I89" t="n">
-        <v>1097.500030517578</v>
+        <v>109750</v>
       </c>
       <c r="J89" t="n">
-        <v>2.112592205104433</v>
+        <v>2.112592172433352</v>
       </c>
       <c r="K89" s="1" t="n">
         <v>46100.625</v>
@@ -3313,10 +3313,10 @@
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>337.3999938964844</v>
+        <v>33740</v>
       </c>
       <c r="I90" t="n">
-        <v>337.3999938964844</v>
+        <v>33740</v>
       </c>
       <c r="J90" t="inlineStr"/>
       <c r="K90" s="1" t="n">
@@ -3343,16 +3343,16 @@
         <v>1</v>
       </c>
       <c r="G91" t="n">
-        <v>814.4000244140625</v>
+        <v>81440</v>
       </c>
       <c r="H91" t="n">
-        <v>337.3999938964844</v>
+        <v>33740</v>
       </c>
       <c r="I91" t="n">
-        <v>1151.800018310547</v>
+        <v>115180</v>
       </c>
       <c r="J91" t="n">
-        <v>2.413752338904676</v>
+        <v>2.413752222880853</v>
       </c>
       <c r="K91" s="1" t="n">
         <v>46100.625</v>
@@ -3377,10 +3377,10 @@
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>313.8999938964844</v>
+        <v>31390</v>
       </c>
       <c r="I92" t="n">
-        <v>313.8999938964844</v>
+        <v>31390</v>
       </c>
       <c r="J92" t="inlineStr"/>
       <c r="K92" s="1" t="n">
@@ -3407,16 +3407,16 @@
         <v>1</v>
       </c>
       <c r="G93" t="n">
-        <v>674.0999755859375</v>
+        <v>67410</v>
       </c>
       <c r="H93" t="n">
-        <v>313.8999938964844</v>
+        <v>31390</v>
       </c>
       <c r="I93" t="n">
-        <v>987.9999694824219</v>
+        <v>98800</v>
       </c>
       <c r="J93" t="n">
-        <v>2.147499167547729</v>
+        <v>2.147499203568015</v>
       </c>
       <c r="K93" s="1" t="n">
         <v>46100.625</v>
@@ -3441,10 +3441,10 @@
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="n">
-        <v>360.2000122070312</v>
+        <v>36020</v>
       </c>
       <c r="I94" t="n">
-        <v>360.2000122070312</v>
+        <v>36020</v>
       </c>
       <c r="J94" t="inlineStr"/>
       <c r="K94" s="1" t="n">
@@ -3471,16 +3471,16 @@
         <v>1</v>
       </c>
       <c r="G95" t="n">
-        <v>585.2000122070312</v>
+        <v>58520</v>
       </c>
       <c r="H95" t="n">
-        <v>360.2000122070312</v>
+        <v>36020</v>
       </c>
       <c r="I95" t="n">
-        <v>945.4000244140625</v>
+        <v>94540</v>
       </c>
       <c r="J95" t="n">
-        <v>1.62465294940267</v>
+        <v>1.624652970571904</v>
       </c>
       <c r="K95" s="1" t="n">
         <v>46100.625</v>
@@ -3505,10 +3505,10 @@
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="n">
-        <v>441.7000122070312</v>
+        <v>44170</v>
       </c>
       <c r="I96" t="n">
-        <v>441.7000122070312</v>
+        <v>44170</v>
       </c>
       <c r="J96" t="inlineStr"/>
       <c r="K96" s="1" t="n">
@@ -3535,16 +3535,16 @@
         <v>1</v>
       </c>
       <c r="G97" t="n">
-        <v>578.9000244140625</v>
+        <v>57890</v>
       </c>
       <c r="H97" t="n">
-        <v>441.7000122070312</v>
+        <v>44170</v>
       </c>
       <c r="I97" t="n">
-        <v>1020.600036621094</v>
+        <v>102060</v>
       </c>
       <c r="J97" t="n">
-        <v>1.310618085613101</v>
+        <v>1.310618066561014</v>
       </c>
       <c r="K97" s="1" t="n">
         <v>46100.625</v>
@@ -3569,10 +3569,10 @@
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="n">
-        <v>504.2000122070312</v>
+        <v>50420</v>
       </c>
       <c r="I98" t="n">
-        <v>504.2000122070312</v>
+        <v>50420</v>
       </c>
       <c r="J98" t="inlineStr"/>
       <c r="K98" s="1" t="n">
@@ -3599,16 +3599,16 @@
         <v>1</v>
       </c>
       <c r="G99" t="n">
-        <v>604.7000122070312</v>
+        <v>60470</v>
       </c>
       <c r="H99" t="n">
-        <v>504.2000122070312</v>
+        <v>50420</v>
       </c>
       <c r="I99" t="n">
-        <v>1108.900024414062</v>
+        <v>110890</v>
       </c>
       <c r="J99" t="n">
-        <v>1.199325659593069</v>
+        <v>1.199325664418881</v>
       </c>
       <c r="K99" s="1" t="n">
         <v>46100.625</v>
@@ -3633,10 +3633,10 @@
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
-        <v>545.2000122070312</v>
+        <v>54520</v>
       </c>
       <c r="I100" t="n">
-        <v>545.2000122070312</v>
+        <v>54520</v>
       </c>
       <c r="J100" t="inlineStr"/>
       <c r="K100" s="1" t="n">
@@ -3663,16 +3663,16 @@
         <v>1</v>
       </c>
       <c r="G101" t="n">
-        <v>611.0999755859375</v>
+        <v>61110</v>
       </c>
       <c r="H101" t="n">
-        <v>545.2000122070312</v>
+        <v>54520</v>
       </c>
       <c r="I101" t="n">
-        <v>1156.299987792969</v>
+        <v>115630</v>
       </c>
       <c r="J101" t="n">
-        <v>1.120873004224882</v>
+        <v>1.120873074101247</v>
       </c>
       <c r="K101" s="1" t="n">
         <v>46100.625</v>
@@ -3697,10 +3697,10 @@
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
-        <v>549</v>
+        <v>54900</v>
       </c>
       <c r="I102" t="n">
-        <v>549</v>
+        <v>54900</v>
       </c>
       <c r="J102" t="inlineStr"/>
       <c r="K102" s="1" t="n">
@@ -3727,16 +3727,16 @@
         <v>1</v>
       </c>
       <c r="G103" t="n">
-        <v>580.5999755859375</v>
+        <v>58060</v>
       </c>
       <c r="H103" t="n">
-        <v>549</v>
+        <v>54900</v>
       </c>
       <c r="I103" t="n">
-        <v>1129.599975585938</v>
+        <v>112960</v>
       </c>
       <c r="J103" t="n">
-        <v>1.057559154072746</v>
+        <v>1.057559198542805</v>
       </c>
       <c r="K103" s="1" t="n">
         <v>46100.625</v>
@@ -3761,10 +3761,10 @@
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>556.7000122070312</v>
+        <v>55670</v>
       </c>
       <c r="I104" t="n">
-        <v>556.7000122070312</v>
+        <v>55670</v>
       </c>
       <c r="J104" t="inlineStr"/>
       <c r="K104" s="1" t="n">
@@ -3791,16 +3791,16 @@
         <v>1</v>
       </c>
       <c r="G105" t="n">
-        <v>528</v>
+        <v>52800</v>
       </c>
       <c r="H105" t="n">
-        <v>556.7000122070312</v>
+        <v>55670</v>
       </c>
       <c r="I105" t="n">
-        <v>1084.700012207031</v>
+        <v>108470</v>
       </c>
       <c r="J105" t="n">
-        <v>0.9484461800292578</v>
+        <v>0.9484462008262978</v>
       </c>
       <c r="K105" s="1" t="n">
         <v>46100.625</v>
@@ -3825,10 +3825,10 @@
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>526.4000244140625</v>
+        <v>52640</v>
       </c>
       <c r="I106" t="n">
-        <v>526.4000244140625</v>
+        <v>52640</v>
       </c>
       <c r="J106" t="inlineStr"/>
       <c r="K106" s="1" t="n">
@@ -3855,16 +3855,16 @@
         <v>1</v>
       </c>
       <c r="G107" t="n">
-        <v>433.5</v>
+        <v>43350</v>
       </c>
       <c r="H107" t="n">
-        <v>526.4000244140625</v>
+        <v>52640</v>
       </c>
       <c r="I107" t="n">
-        <v>959.9000244140625</v>
+        <v>95990</v>
       </c>
       <c r="J107" t="n">
-        <v>0.8235181988878708</v>
+        <v>0.8235182370820668</v>
       </c>
       <c r="K107" s="1" t="n">
         <v>46100.625</v>
@@ -3889,10 +3889,10 @@
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="n">
-        <v>415.2000122070312</v>
+        <v>41520</v>
       </c>
       <c r="I108" t="n">
-        <v>415.2000122070312</v>
+        <v>41520</v>
       </c>
       <c r="J108" t="inlineStr"/>
       <c r="K108" s="1" t="n">
@@ -3919,16 +3919,16 @@
         <v>1</v>
       </c>
       <c r="G109" t="n">
-        <v>354.3999938964844</v>
+        <v>35440</v>
       </c>
       <c r="H109" t="n">
-        <v>415.2000122070312</v>
+        <v>41520</v>
       </c>
       <c r="I109" t="n">
-        <v>769.6000061035156</v>
+        <v>76960</v>
       </c>
       <c r="J109" t="n">
-        <v>0.8535645074108761</v>
+        <v>0.8535645472061657</v>
       </c>
       <c r="K109" s="1" t="n">
         <v>46100.625</v>
@@ -3953,10 +3953,10 @@
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="n">
-        <v>318.3999938964844</v>
+        <v>31840</v>
       </c>
       <c r="I110" t="n">
-        <v>318.3999938964844</v>
+        <v>31840</v>
       </c>
       <c r="J110" t="inlineStr"/>
       <c r="K110" s="1" t="n">
@@ -3983,16 +3983,16 @@
         <v>1</v>
       </c>
       <c r="G111" t="n">
-        <v>303.6000061035156</v>
+        <v>30360</v>
       </c>
       <c r="H111" t="n">
-        <v>318.3999938964844</v>
+        <v>31840</v>
       </c>
       <c r="I111" t="n">
-        <v>622</v>
+        <v>62200</v>
       </c>
       <c r="J111" t="n">
-        <v>0.9535176253873283</v>
+        <v>0.9535175879396985</v>
       </c>
       <c r="K111" s="1" t="n">
         <v>46100.625</v>
@@ -4017,10 +4017,10 @@
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="n">
-        <v>272.5</v>
+        <v>27250</v>
       </c>
       <c r="I112" t="n">
-        <v>272.5</v>
+        <v>27250</v>
       </c>
       <c r="J112" t="inlineStr"/>
       <c r="K112" s="1" t="n">
@@ -4047,16 +4047,16 @@
         <v>1</v>
       </c>
       <c r="G113" t="n">
-        <v>268.7999877929688</v>
+        <v>26880</v>
       </c>
       <c r="H113" t="n">
-        <v>272.5</v>
+        <v>27250</v>
       </c>
       <c r="I113" t="n">
-        <v>541.2999877929688</v>
+        <v>54130</v>
       </c>
       <c r="J113" t="n">
-        <v>0.9864219735521789</v>
+        <v>0.9864220183486239</v>
       </c>
       <c r="K113" s="1" t="n">
         <v>46100.625</v>
@@ -4081,10 +4081,10 @@
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="n">
-        <v>293.6000061035156</v>
+        <v>29360</v>
       </c>
       <c r="I114" t="n">
-        <v>293.6000061035156</v>
+        <v>29360</v>
       </c>
       <c r="J114" t="inlineStr"/>
       <c r="K114" s="1" t="n">
@@ -4111,16 +4111,16 @@
         <v>1</v>
       </c>
       <c r="G115" t="n">
-        <v>298.6000061035156</v>
+        <v>29860</v>
       </c>
       <c r="H115" t="n">
-        <v>293.6000061035156</v>
+        <v>29360</v>
       </c>
       <c r="I115" t="n">
-        <v>592.2000122070312</v>
+        <v>59220</v>
       </c>
       <c r="J115" t="n">
-        <v>1.017029972398015</v>
+        <v>1.017029972752044</v>
       </c>
       <c r="K115" s="1" t="n">
         <v>46100.625</v>
@@ -4145,10 +4145,10 @@
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="n">
-        <v>347.2999877929688</v>
+        <v>34730</v>
       </c>
       <c r="I116" t="n">
-        <v>347.2999877929688</v>
+        <v>34730</v>
       </c>
       <c r="J116" t="inlineStr"/>
       <c r="K116" s="1" t="n">
@@ -4175,16 +4175,16 @@
         <v>1</v>
       </c>
       <c r="G117" t="n">
-        <v>343.5</v>
+        <v>34350</v>
       </c>
       <c r="H117" t="n">
-        <v>347.2999877929688</v>
+        <v>34730</v>
       </c>
       <c r="I117" t="n">
-        <v>690.7999877929688</v>
+        <v>69080</v>
       </c>
       <c r="J117" t="n">
-        <v>0.9890584856707971</v>
+        <v>0.9890584509069968</v>
       </c>
       <c r="K117" s="1" t="n">
         <v>46100.625</v>
@@ -4209,10 +4209,10 @@
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="n">
-        <v>374.7000122070312</v>
+        <v>37470</v>
       </c>
       <c r="I118" t="n">
-        <v>374.7000122070312</v>
+        <v>37470</v>
       </c>
       <c r="J118" t="inlineStr"/>
       <c r="K118" s="1" t="n">
@@ -4239,16 +4239,16 @@
         <v>1</v>
       </c>
       <c r="G119" t="n">
-        <v>355.6000061035156</v>
+        <v>35560</v>
       </c>
       <c r="H119" t="n">
-        <v>374.7000122070312</v>
+        <v>37470</v>
       </c>
       <c r="I119" t="n">
-        <v>730.3000183105469</v>
+        <v>73030</v>
       </c>
       <c r="J119" t="n">
-        <v>0.9490258727481375</v>
+        <v>0.9490258873765679</v>
       </c>
       <c r="K119" s="1" t="n">
         <v>46100.625</v>
@@ -4273,10 +4273,10 @@
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="n">
-        <v>392.2999877929688</v>
+        <v>39230</v>
       </c>
       <c r="I120" t="n">
-        <v>392.2999877929688</v>
+        <v>39230</v>
       </c>
       <c r="J120" t="inlineStr"/>
       <c r="K120" s="1" t="n">
@@ -4303,16 +4303,16 @@
         <v>1</v>
       </c>
       <c r="G121" t="n">
-        <v>371</v>
+        <v>37100</v>
       </c>
       <c r="H121" t="n">
-        <v>392.2999877929688</v>
+        <v>39230</v>
       </c>
       <c r="I121" t="n">
-        <v>763.2999877929688</v>
+        <v>76330</v>
       </c>
       <c r="J121" t="n">
-        <v>0.9457048471686175</v>
+        <v>0.9457048177415244</v>
       </c>
       <c r="K121" s="1" t="n">
         <v>46100.625</v>
@@ -4337,10 +4337,10 @@
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>417.6000061035156</v>
+        <v>41760</v>
       </c>
       <c r="I122" t="n">
-        <v>417.6000061035156</v>
+        <v>41760</v>
       </c>
       <c r="J122" t="inlineStr"/>
       <c r="K122" s="1" t="n">
@@ -4367,16 +4367,16 @@
         <v>1</v>
       </c>
       <c r="G123" t="n">
-        <v>392.2000122070312</v>
+        <v>39220</v>
       </c>
       <c r="H123" t="n">
-        <v>417.6000061035156</v>
+        <v>41760</v>
       </c>
       <c r="I123" t="n">
-        <v>809.8000183105469</v>
+        <v>80980</v>
       </c>
       <c r="J123" t="n">
-        <v>0.9391762607154077</v>
+        <v>0.939176245210728</v>
       </c>
       <c r="K123" s="1" t="n">
         <v>46100.625</v>
@@ -4401,10 +4401,10 @@
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="n">
-        <v>405.7000122070312</v>
+        <v>40570</v>
       </c>
       <c r="I124" t="n">
-        <v>405.7000122070312</v>
+        <v>40570</v>
       </c>
       <c r="J124" t="inlineStr"/>
       <c r="K124" s="1" t="n">
@@ -4431,16 +4431,16 @@
         <v>1</v>
       </c>
       <c r="G125" t="n">
-        <v>366.6000061035156</v>
+        <v>36660</v>
       </c>
       <c r="H125" t="n">
-        <v>405.7000122070312</v>
+        <v>40570</v>
       </c>
       <c r="I125" t="n">
-        <v>772.3000183105469</v>
+        <v>77230</v>
       </c>
       <c r="J125" t="n">
-        <v>0.903623354875418</v>
+        <v>0.9036233670199655</v>
       </c>
       <c r="K125" s="1" t="n">
         <v>46100.625</v>
@@ -4465,10 +4465,10 @@
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="n">
-        <v>339.3999938964844</v>
+        <v>33940</v>
       </c>
       <c r="I126" t="n">
-        <v>339.3999938964844</v>
+        <v>33940</v>
       </c>
       <c r="J126" t="inlineStr"/>
       <c r="K126" s="1" t="n">
@@ -4495,16 +4495,16 @@
         <v>1</v>
       </c>
       <c r="G127" t="n">
-        <v>310.7000122070312</v>
+        <v>31070</v>
       </c>
       <c r="H127" t="n">
-        <v>339.3999938964844</v>
+        <v>33940</v>
       </c>
       <c r="I127" t="n">
-        <v>650.1000061035156</v>
+        <v>65010</v>
       </c>
       <c r="J127" t="n">
-        <v>0.9154390624467527</v>
+        <v>0.9154390100176782</v>
       </c>
       <c r="K127" s="1" t="n">
         <v>46100.625</v>
@@ -4529,10 +4529,10 @@
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>262.7000122070312</v>
+        <v>26270</v>
       </c>
       <c r="I128" t="n">
-        <v>262.7000122070312</v>
+        <v>26270</v>
       </c>
       <c r="J128" t="inlineStr"/>
       <c r="K128" s="1" t="n">
@@ -4559,16 +4559,16 @@
         <v>1</v>
       </c>
       <c r="G129" t="n">
-        <v>259.7000122070312</v>
+        <v>25970</v>
       </c>
       <c r="H129" t="n">
-        <v>262.7000122070312</v>
+        <v>26270</v>
       </c>
       <c r="I129" t="n">
-        <v>522.4000244140625</v>
+        <v>52240</v>
       </c>
       <c r="J129" t="n">
-        <v>0.9885801299558535</v>
+        <v>0.9885801294251998</v>
       </c>
       <c r="K129" s="1" t="n">
         <v>46100.625</v>
@@ -4593,10 +4593,10 @@
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="n">
-        <v>213.8999938964844</v>
+        <v>21390</v>
       </c>
       <c r="I130" t="n">
-        <v>213.8999938964844</v>
+        <v>21390</v>
       </c>
       <c r="J130" t="inlineStr"/>
       <c r="K130" s="1" t="n">
@@ -4623,16 +4623,16 @@
         <v>1</v>
       </c>
       <c r="G131" t="n">
-        <v>226.8000030517578</v>
+        <v>22680</v>
       </c>
       <c r="H131" t="n">
-        <v>213.8999938964844</v>
+        <v>21390</v>
       </c>
       <c r="I131" t="n">
-        <v>440.6999969482422</v>
+        <v>44070</v>
       </c>
       <c r="J131" t="n">
-        <v>1.060308599922244</v>
+        <v>1.06030855539972</v>
       </c>
       <c r="K131" s="1" t="n">
         <v>46100.625</v>
@@ -4657,10 +4657,10 @@
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>211.3000030517578</v>
+        <v>21130</v>
       </c>
       <c r="I132" t="n">
-        <v>211.3000030517578</v>
+        <v>21130</v>
       </c>
       <c r="J132" t="inlineStr"/>
       <c r="K132" s="1" t="n">
@@ -4687,16 +4687,16 @@
         <v>1</v>
       </c>
       <c r="G133" t="n">
-        <v>228</v>
+        <v>22800</v>
       </c>
       <c r="H133" t="n">
-        <v>211.3000030517578</v>
+        <v>21130</v>
       </c>
       <c r="I133" t="n">
-        <v>439.3000030517578</v>
+        <v>43930</v>
       </c>
       <c r="J133" t="n">
-        <v>1.079034532451718</v>
+        <v>1.079034548035968</v>
       </c>
       <c r="K133" s="1" t="n">
         <v>46100.625</v>
@@ -4721,10 +4721,10 @@
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>230.1000061035156</v>
+        <v>23010</v>
       </c>
       <c r="I134" t="n">
-        <v>230.1000061035156</v>
+        <v>23010</v>
       </c>
       <c r="J134" t="inlineStr"/>
       <c r="K134" s="1" t="n">
@@ -4751,16 +4751,16 @@
         <v>1</v>
       </c>
       <c r="G135" t="n">
-        <v>244.5</v>
+        <v>24450</v>
       </c>
       <c r="H135" t="n">
-        <v>230.1000061035156</v>
+        <v>23010</v>
       </c>
       <c r="I135" t="n">
-        <v>474.6000061035156</v>
+        <v>47460</v>
       </c>
       <c r="J135" t="n">
-        <v>1.062581458124804</v>
+        <v>1.0625814863103</v>
       </c>
       <c r="K135" s="1" t="n">
         <v>46100.625</v>
@@ -4785,10 +4785,10 @@
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="n">
-        <v>232.5</v>
+        <v>23250</v>
       </c>
       <c r="I136" t="n">
-        <v>232.5</v>
+        <v>23250</v>
       </c>
       <c r="J136" t="inlineStr"/>
       <c r="K136" s="1" t="n">
@@ -4815,13 +4815,13 @@
         <v>1</v>
       </c>
       <c r="G137" t="n">
-        <v>248</v>
+        <v>24800</v>
       </c>
       <c r="H137" t="n">
-        <v>232.5</v>
+        <v>23250</v>
       </c>
       <c r="I137" t="n">
-        <v>480.5</v>
+        <v>48050</v>
       </c>
       <c r="J137" t="n">
         <v>1.066666666666667</v>
@@ -4849,10 +4849,10 @@
       </c>
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="n">
-        <v>222.3000030517578</v>
+        <v>22230</v>
       </c>
       <c r="I138" t="n">
-        <v>222.3000030517578</v>
+        <v>22230</v>
       </c>
       <c r="J138" t="inlineStr"/>
       <c r="K138" s="1" t="n">
@@ -4879,16 +4879,16 @@
         <v>1</v>
       </c>
       <c r="G139" t="n">
-        <v>229.8000030517578</v>
+        <v>22980</v>
       </c>
       <c r="H139" t="n">
-        <v>222.3000030517578</v>
+        <v>22230</v>
       </c>
       <c r="I139" t="n">
-        <v>452.1000061035156</v>
+        <v>45210</v>
       </c>
       <c r="J139" t="n">
-        <v>1.033738191169767</v>
+        <v>1.033738191632928</v>
       </c>
       <c r="K139" s="1" t="n">
         <v>46100.625</v>
@@ -4913,10 +4913,10 @@
       </c>
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="n">
-        <v>208.6000061035156</v>
+        <v>20860</v>
       </c>
       <c r="I140" t="n">
-        <v>208.6000061035156</v>
+        <v>20860</v>
       </c>
       <c r="J140" t="inlineStr"/>
       <c r="K140" s="1" t="n">
@@ -4943,16 +4943,16 @@
         <v>1</v>
       </c>
       <c r="G141" t="n">
-        <v>209.8999938964844</v>
+        <v>20990</v>
       </c>
       <c r="H141" t="n">
-        <v>208.6000061035156</v>
+        <v>20860</v>
       </c>
       <c r="I141" t="n">
-        <v>418.5</v>
+        <v>41850</v>
       </c>
       <c r="J141" t="n">
-        <v>1.006231964309357</v>
+        <v>1.006232023010547</v>
       </c>
       <c r="K141" s="1" t="n">
         <v>46100.625</v>
@@ -4977,10 +4977,10 @@
       </c>
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="n">
-        <v>191</v>
+        <v>19100</v>
       </c>
       <c r="I142" t="n">
-        <v>191</v>
+        <v>19100</v>
       </c>
       <c r="J142" t="inlineStr"/>
       <c r="K142" s="1" t="n">
@@ -5007,16 +5007,16 @@
         <v>1</v>
       </c>
       <c r="G143" t="n">
-        <v>195.1000061035156</v>
+        <v>19510</v>
       </c>
       <c r="H143" t="n">
-        <v>191</v>
+        <v>19100</v>
       </c>
       <c r="I143" t="n">
-        <v>386.1000061035156</v>
+        <v>38610</v>
       </c>
       <c r="J143" t="n">
-        <v>1.021466000541967</v>
+        <v>1.021465968586387</v>
       </c>
       <c r="K143" s="1" t="n">
         <v>46100.625</v>
@@ -5041,10 +5041,10 @@
       </c>
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="n">
-        <v>187.6999969482422</v>
+        <v>18770</v>
       </c>
       <c r="I144" t="n">
-        <v>187.6999969482422</v>
+        <v>18770</v>
       </c>
       <c r="J144" t="inlineStr"/>
       <c r="K144" s="1" t="n">
@@ -5071,16 +5071,16 @@
         <v>1</v>
       </c>
       <c r="G145" t="n">
-        <v>186.3000030517578</v>
+        <v>18630</v>
       </c>
       <c r="H145" t="n">
-        <v>187.6999969482422</v>
+        <v>18770</v>
       </c>
       <c r="I145" t="n">
-        <v>374</v>
+        <v>37400</v>
       </c>
       <c r="J145" t="n">
-        <v>0.9925413216875522</v>
+        <v>0.9925412892914225</v>
       </c>
       <c r="K145" s="1" t="n">
         <v>46100.625</v>
@@ -5105,10 +5105,10 @@
       </c>
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="n">
-        <v>194.3000030517578</v>
+        <v>19430</v>
       </c>
       <c r="I146" t="n">
-        <v>194.3000030517578</v>
+        <v>19430</v>
       </c>
       <c r="J146" t="inlineStr"/>
       <c r="K146" s="1" t="n">
@@ -5135,16 +5135,16 @@
         <v>1</v>
       </c>
       <c r="G147" t="n">
-        <v>180.8999938964844</v>
+        <v>18090</v>
       </c>
       <c r="H147" t="n">
-        <v>194.3000030517578</v>
+        <v>19430</v>
       </c>
       <c r="I147" t="n">
-        <v>375.1999969482422</v>
+        <v>37520</v>
       </c>
       <c r="J147" t="n">
-        <v>0.9310344367225567</v>
+        <v>0.9310344827586207</v>
       </c>
       <c r="K147" s="1" t="n">
         <v>46100.625</v>
@@ -5169,10 +5169,10 @@
       </c>
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="n">
-        <v>194.3000030517578</v>
+        <v>19430</v>
       </c>
       <c r="I148" t="n">
-        <v>194.3000030517578</v>
+        <v>19430</v>
       </c>
       <c r="J148" t="inlineStr"/>
       <c r="K148" s="1" t="n">
@@ -5199,16 +5199,16 @@
         <v>1</v>
       </c>
       <c r="G149" t="n">
-        <v>183.1999969482422</v>
+        <v>18320</v>
       </c>
       <c r="H149" t="n">
-        <v>194.3000030517578</v>
+        <v>19430</v>
       </c>
       <c r="I149" t="n">
-        <v>377.5</v>
+        <v>37750</v>
       </c>
       <c r="J149" t="n">
-        <v>0.9428718171426956</v>
+        <v>0.9428718476582604</v>
       </c>
       <c r="K149" s="1" t="n">
         <v>46100.625</v>
@@ -5233,10 +5233,10 @@
       </c>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="n">
-        <v>192.3000030517578</v>
+        <v>19230</v>
       </c>
       <c r="I150" t="n">
-        <v>192.3000030517578</v>
+        <v>19230</v>
       </c>
       <c r="J150" t="inlineStr"/>
       <c r="K150" s="1" t="n">
@@ -5263,16 +5263,16 @@
         <v>1</v>
       </c>
       <c r="G151" t="n">
-        <v>193.6999969482422</v>
+        <v>19370</v>
       </c>
       <c r="H151" t="n">
-        <v>192.3000030517578</v>
+        <v>19230</v>
       </c>
       <c r="I151" t="n">
-        <v>386</v>
+        <v>38600</v>
       </c>
       <c r="J151" t="n">
-        <v>1.007280259356562</v>
+        <v>1.007280291211649</v>
       </c>
       <c r="K151" s="1" t="n">
         <v>46100.625</v>
@@ -5297,10 +5297,10 @@
       </c>
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="n">
-        <v>186.8000030517578</v>
+        <v>18680</v>
       </c>
       <c r="I152" t="n">
-        <v>186.8000030517578</v>
+        <v>18680</v>
       </c>
       <c r="J152" t="inlineStr"/>
       <c r="K152" s="1" t="n">
@@ -5327,16 +5327,16 @@
         <v>1</v>
       </c>
       <c r="G153" t="n">
-        <v>193.3999938964844</v>
+        <v>19340</v>
       </c>
       <c r="H153" t="n">
-        <v>186.8000030517578</v>
+        <v>18680</v>
       </c>
       <c r="I153" t="n">
-        <v>380.1999969482422</v>
+        <v>38020</v>
       </c>
       <c r="J153" t="n">
-        <v>1.035331856193267</v>
+        <v>1.035331905781585</v>
       </c>
       <c r="K153" s="1" t="n">
         <v>46100.625</v>
@@ -5361,10 +5361,10 @@
       </c>
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="n">
-        <v>178.1000061035156</v>
+        <v>17810</v>
       </c>
       <c r="I154" t="n">
-        <v>178.1000061035156</v>
+        <v>17810</v>
       </c>
       <c r="J154" t="inlineStr"/>
       <c r="K154" s="1" t="n">
@@ -5391,16 +5391,16 @@
         <v>1</v>
       </c>
       <c r="G155" t="n">
-        <v>182.8000030517578</v>
+        <v>18280</v>
       </c>
       <c r="H155" t="n">
-        <v>178.1000061035156</v>
+        <v>17810</v>
       </c>
       <c r="I155" t="n">
-        <v>360.9000091552734</v>
+        <v>36090</v>
       </c>
       <c r="J155" t="n">
-        <v>1.026389650685977</v>
+        <v>1.026389668725435</v>
       </c>
       <c r="K155" s="1" t="n">
         <v>46100.625</v>
@@ -5425,10 +5425,10 @@
       </c>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="n">
-        <v>176.8999938964844</v>
+        <v>17690</v>
       </c>
       <c r="I156" t="n">
-        <v>176.8999938964844</v>
+        <v>17690</v>
       </c>
       <c r="J156" t="inlineStr"/>
       <c r="K156" s="1" t="n">
@@ -5455,16 +5455,16 @@
         <v>1</v>
       </c>
       <c r="G157" t="n">
-        <v>177.8000030517578</v>
+        <v>17780</v>
       </c>
       <c r="H157" t="n">
-        <v>176.8999938964844</v>
+        <v>17690</v>
       </c>
       <c r="I157" t="n">
-        <v>354.6999969482422</v>
+        <v>35470</v>
       </c>
       <c r="J157" t="n">
-        <v>1.00508767205385</v>
+        <v>1.005087620124364</v>
       </c>
       <c r="K157" s="1" t="n">
         <v>46100.625</v>
@@ -5489,10 +5489,10 @@
       </c>
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="n">
-        <v>184</v>
+        <v>18400</v>
       </c>
       <c r="I158" t="n">
-        <v>184</v>
+        <v>18400</v>
       </c>
       <c r="J158" t="inlineStr"/>
       <c r="K158" s="1" t="n">
@@ -5519,16 +5519,16 @@
         <v>1</v>
       </c>
       <c r="G159" t="n">
-        <v>179.1999969482422</v>
+        <v>17920</v>
       </c>
       <c r="H159" t="n">
-        <v>184</v>
+        <v>18400</v>
       </c>
       <c r="I159" t="n">
-        <v>363.1999969482422</v>
+        <v>36320</v>
       </c>
       <c r="J159" t="n">
-        <v>0.9739130268926206</v>
+        <v>0.9739130434782609</v>
       </c>
       <c r="K159" s="1" t="n">
         <v>46100.625</v>
@@ -5553,10 +5553,10 @@
       </c>
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="n">
-        <v>187</v>
+        <v>18700</v>
       </c>
       <c r="I160" t="n">
-        <v>187</v>
+        <v>18700</v>
       </c>
       <c r="J160" t="inlineStr"/>
       <c r="K160" s="1" t="n">
@@ -5583,13 +5583,13 @@
         <v>1</v>
       </c>
       <c r="G161" t="n">
-        <v>184.5</v>
+        <v>18450</v>
       </c>
       <c r="H161" t="n">
-        <v>187</v>
+        <v>18700</v>
       </c>
       <c r="I161" t="n">
-        <v>371.5</v>
+        <v>37150</v>
       </c>
       <c r="J161" t="n">
         <v>0.9866310160427807</v>
@@ -5617,10 +5617,10 @@
       </c>
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="n">
-        <v>192.6000061035156</v>
+        <v>19260</v>
       </c>
       <c r="I162" t="n">
-        <v>192.6000061035156</v>
+        <v>19260</v>
       </c>
       <c r="J162" t="inlineStr"/>
       <c r="K162" s="1" t="n">
@@ -5647,16 +5647,16 @@
         <v>1</v>
       </c>
       <c r="G163" t="n">
-        <v>191.8999938964844</v>
+        <v>19190</v>
       </c>
       <c r="H163" t="n">
-        <v>192.6000061035156</v>
+        <v>19260</v>
       </c>
       <c r="I163" t="n">
-        <v>384.5</v>
+        <v>38450</v>
       </c>
       <c r="J163" t="n">
-        <v>0.996365461137862</v>
+        <v>0.9963655244029076</v>
       </c>
       <c r="K163" s="1" t="n">
         <v>46100.625</v>
@@ -5681,10 +5681,10 @@
       </c>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="n">
-        <v>194.1000061035156</v>
+        <v>19410</v>
       </c>
       <c r="I164" t="n">
-        <v>194.1000061035156</v>
+        <v>19410</v>
       </c>
       <c r="J164" t="inlineStr"/>
       <c r="K164" s="1" t="n">
@@ -5711,16 +5711,16 @@
         <v>1</v>
       </c>
       <c r="G165" t="n">
-        <v>192</v>
+        <v>19200</v>
       </c>
       <c r="H165" t="n">
-        <v>194.1000061035156</v>
+        <v>19410</v>
       </c>
       <c r="I165" t="n">
-        <v>386.1000061035156</v>
+        <v>38610</v>
       </c>
       <c r="J165" t="n">
-        <v>0.9891808035163293</v>
+        <v>0.9891808346213292</v>
       </c>
       <c r="K165" s="1" t="n">
         <v>46100.625</v>
@@ -5745,10 +5745,10 @@
       </c>
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="n">
-        <v>182.3999938964844</v>
+        <v>18240</v>
       </c>
       <c r="I166" t="n">
-        <v>182.3999938964844</v>
+        <v>18240</v>
       </c>
       <c r="J166" t="inlineStr"/>
       <c r="K166" s="1" t="n">
@@ -5775,16 +5775,16 @@
         <v>1</v>
       </c>
       <c r="G167" t="n">
-        <v>188.3000030517578</v>
+        <v>18830</v>
       </c>
       <c r="H167" t="n">
-        <v>182.3999938964844</v>
+        <v>18240</v>
       </c>
       <c r="I167" t="n">
-        <v>370.6999969482422</v>
+        <v>37070</v>
       </c>
       <c r="J167" t="n">
-        <v>1.032346542503844</v>
+        <v>1.03234649122807</v>
       </c>
       <c r="K167" s="1" t="n">
         <v>46100.625</v>
@@ -5809,10 +5809,10 @@
       </c>
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="n">
-        <v>172.6999969482422</v>
+        <v>17270</v>
       </c>
       <c r="I168" t="n">
-        <v>172.6999969482422</v>
+        <v>17270</v>
       </c>
       <c r="J168" t="inlineStr"/>
       <c r="K168" s="1" t="n">
@@ -5839,16 +5839,16 @@
         <v>1</v>
       </c>
       <c r="G169" t="n">
-        <v>185.6000061035156</v>
+        <v>18560</v>
       </c>
       <c r="H169" t="n">
-        <v>172.6999969482422</v>
+        <v>17270</v>
       </c>
       <c r="I169" t="n">
-        <v>358.3000030517578</v>
+        <v>35830</v>
       </c>
       <c r="J169" t="n">
-        <v>1.074696058964839</v>
+        <v>1.07469600463231</v>
       </c>
       <c r="K169" s="1" t="n">
         <v>46100.625</v>
@@ -5873,10 +5873,10 @@
       </c>
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="n">
-        <v>165.8000030517578</v>
+        <v>16580</v>
       </c>
       <c r="I170" t="n">
-        <v>165.8000030517578</v>
+        <v>16580</v>
       </c>
       <c r="J170" t="inlineStr"/>
       <c r="K170" s="1" t="n">
@@ -5903,16 +5903,16 @@
         <v>1</v>
       </c>
       <c r="G171" t="n">
-        <v>183.6000061035156</v>
+        <v>18360</v>
       </c>
       <c r="H171" t="n">
-        <v>165.8000030517578</v>
+        <v>16580</v>
       </c>
       <c r="I171" t="n">
-        <v>349.4000091552734</v>
+        <v>34940</v>
       </c>
       <c r="J171" t="n">
-        <v>1.107358279397626</v>
+        <v>1.107358262967431</v>
       </c>
       <c r="K171" s="1" t="n">
         <v>46100.625</v>
@@ -5937,10 +5937,10 @@
       </c>
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="n">
-        <v>162.3000030517578</v>
+        <v>16230</v>
       </c>
       <c r="I172" t="n">
-        <v>162.3000030517578</v>
+        <v>16230</v>
       </c>
       <c r="J172" t="inlineStr"/>
       <c r="K172" s="1" t="n">
@@ -5967,16 +5967,16 @@
         <v>1</v>
       </c>
       <c r="G173" t="n">
-        <v>186.8999938964844</v>
+        <v>18690</v>
       </c>
       <c r="H173" t="n">
-        <v>162.3000030517578</v>
+        <v>16230</v>
       </c>
       <c r="I173" t="n">
-        <v>349.1999969482422</v>
+        <v>34920</v>
       </c>
       <c r="J173" t="n">
-        <v>1.151571105250575</v>
+        <v>1.151571164510166</v>
       </c>
       <c r="K173" s="1" t="n">
         <v>46100.625</v>
@@ -6001,10 +6001,10 @@
       </c>
       <c r="G174" t="inlineStr"/>
       <c r="H174" t="n">
-        <v>166.6999969482422</v>
+        <v>16670</v>
       </c>
       <c r="I174" t="n">
-        <v>166.6999969482422</v>
+        <v>16670</v>
       </c>
       <c r="J174" t="inlineStr"/>
       <c r="K174" s="1" t="n">
@@ -6031,16 +6031,16 @@
         <v>1</v>
       </c>
       <c r="G175" t="n">
-        <v>190.5</v>
+        <v>19050</v>
       </c>
       <c r="H175" t="n">
-        <v>166.6999969482422</v>
+        <v>16670</v>
       </c>
       <c r="I175" t="n">
-        <v>357.1999969482422</v>
+        <v>35720</v>
       </c>
       <c r="J175" t="n">
-        <v>1.142771466631444</v>
+        <v>1.142771445710858</v>
       </c>
       <c r="K175" s="1" t="n">
         <v>46100.625</v>
@@ -6065,10 +6065,10 @@
       </c>
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="n">
-        <v>171</v>
+        <v>17100</v>
       </c>
       <c r="I176" t="n">
-        <v>171</v>
+        <v>17100</v>
       </c>
       <c r="J176" t="inlineStr"/>
       <c r="K176" s="1" t="n">
@@ -6095,16 +6095,16 @@
         <v>1</v>
       </c>
       <c r="G177" t="n">
-        <v>190.6999969482422</v>
+        <v>19070</v>
       </c>
       <c r="H177" t="n">
-        <v>171</v>
+        <v>17100</v>
       </c>
       <c r="I177" t="n">
-        <v>361.6999969482422</v>
+        <v>36170</v>
       </c>
       <c r="J177" t="n">
-        <v>1.115204660516036</v>
+        <v>1.115204678362573</v>
       </c>
       <c r="K177" s="1" t="n">
         <v>46100.625</v>
@@ -6129,10 +6129,10 @@
       </c>
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="n">
-        <v>175.1000061035156</v>
+        <v>17510</v>
       </c>
       <c r="I178" t="n">
-        <v>175.1000061035156</v>
+        <v>17510</v>
       </c>
       <c r="J178" t="inlineStr"/>
       <c r="K178" s="1" t="n">
@@ -6159,16 +6159,16 @@
         <v>1</v>
       </c>
       <c r="G179" t="n">
-        <v>193.8999938964844</v>
+        <v>19390</v>
       </c>
       <c r="H179" t="n">
-        <v>175.1000061035156</v>
+        <v>17510</v>
       </c>
       <c r="I179" t="n">
-        <v>369</v>
+        <v>36900</v>
       </c>
       <c r="J179" t="n">
-        <v>1.107367145274995</v>
+        <v>1.107367218732153</v>
       </c>
       <c r="K179" s="1" t="n">
         <v>46100.625</v>
@@ -6193,10 +6193,10 @@
       </c>
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="n">
-        <v>177.6999969482422</v>
+        <v>17770</v>
       </c>
       <c r="I180" t="n">
-        <v>177.6999969482422</v>
+        <v>17770</v>
       </c>
       <c r="J180" t="inlineStr"/>
       <c r="K180" s="1" t="n">
@@ -6223,16 +6223,16 @@
         <v>1</v>
       </c>
       <c r="G181" t="n">
-        <v>198.3000030517578</v>
+        <v>19830</v>
       </c>
       <c r="H181" t="n">
-        <v>177.6999969482422</v>
+        <v>17770</v>
       </c>
       <c r="I181" t="n">
-        <v>376</v>
+        <v>37600</v>
       </c>
       <c r="J181" t="n">
-        <v>1.115925753839578</v>
+        <v>1.115925717501407</v>
       </c>
       <c r="K181" s="1" t="n">
         <v>46100.625</v>
@@ -6257,10 +6257,10 @@
       </c>
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="n">
-        <v>173.6000061035156</v>
+        <v>17360</v>
       </c>
       <c r="I182" t="n">
-        <v>173.6000061035156</v>
+        <v>17360</v>
       </c>
       <c r="J182" t="inlineStr"/>
       <c r="K182" s="1" t="n">
@@ -6287,16 +6287,16 @@
         <v>1</v>
       </c>
       <c r="G183" t="n">
-        <v>198</v>
+        <v>19800</v>
       </c>
       <c r="H183" t="n">
-        <v>173.6000061035156</v>
+        <v>17360</v>
       </c>
       <c r="I183" t="n">
-        <v>371.6000061035156</v>
+        <v>37160</v>
       </c>
       <c r="J183" t="n">
-        <v>1.140552955291574</v>
+        <v>1.140552995391705</v>
       </c>
       <c r="K183" s="1" t="n">
         <v>46100.625</v>
@@ -6321,10 +6321,10 @@
       </c>
       <c r="G184" t="inlineStr"/>
       <c r="H184" t="n">
-        <v>178.8000030517578</v>
+        <v>17880</v>
       </c>
       <c r="I184" t="n">
-        <v>178.8000030517578</v>
+        <v>17880</v>
       </c>
       <c r="J184" t="inlineStr"/>
       <c r="K184" s="1" t="n">
@@ -6351,16 +6351,16 @@
         <v>1</v>
       </c>
       <c r="G185" t="n">
-        <v>194.6000061035156</v>
+        <v>19460</v>
       </c>
       <c r="H185" t="n">
-        <v>178.8000030517578</v>
+        <v>17880</v>
       </c>
       <c r="I185" t="n">
-        <v>373.4000091552734</v>
+        <v>37340</v>
       </c>
       <c r="J185" t="n">
-        <v>1.088366905940064</v>
+        <v>1.088366890380313</v>
       </c>
       <c r="K185" s="1" t="n">
         <v>46100.625</v>
@@ -6385,10 +6385,10 @@
       </c>
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="n">
-        <v>194</v>
+        <v>19400</v>
       </c>
       <c r="I186" t="n">
-        <v>194</v>
+        <v>19400</v>
       </c>
       <c r="J186" t="inlineStr"/>
       <c r="K186" s="1" t="n">
@@ -6415,16 +6415,16 @@
         <v>1</v>
       </c>
       <c r="G187" t="n">
-        <v>191.1999969482422</v>
+        <v>19120</v>
       </c>
       <c r="H187" t="n">
-        <v>194</v>
+        <v>19400</v>
       </c>
       <c r="I187" t="n">
-        <v>385.1999969482422</v>
+        <v>38520</v>
       </c>
       <c r="J187" t="n">
-        <v>0.985566994578568</v>
+        <v>0.9855670103092784</v>
       </c>
       <c r="K187" s="1" t="n">
         <v>46100.625</v>
@@ -6449,10 +6449,10 @@
       </c>
       <c r="G188" t="inlineStr"/>
       <c r="H188" t="n">
-        <v>201.1000061035156</v>
+        <v>20110</v>
       </c>
       <c r="I188" t="n">
-        <v>201.1000061035156</v>
+        <v>20110</v>
       </c>
       <c r="J188" t="inlineStr"/>
       <c r="K188" s="1" t="n">
@@ -6479,16 +6479,16 @@
         <v>1</v>
       </c>
       <c r="G189" t="n">
-        <v>193.1000061035156</v>
+        <v>19310</v>
       </c>
       <c r="H189" t="n">
-        <v>201.1000061035156</v>
+        <v>20110</v>
       </c>
       <c r="I189" t="n">
-        <v>394.2000122070312</v>
+        <v>39420</v>
       </c>
       <c r="J189" t="n">
-        <v>0.9602187978259831</v>
+        <v>0.9602187966185977</v>
       </c>
       <c r="K189" s="1" t="n">
         <v>46100.625</v>
@@ -6513,10 +6513,10 @@
       </c>
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="n">
-        <v>202.3999938964844</v>
+        <v>20240</v>
       </c>
       <c r="I190" t="n">
-        <v>202.3999938964844</v>
+        <v>20240</v>
       </c>
       <c r="J190" t="inlineStr"/>
       <c r="K190" s="1" t="n">
@@ -6543,16 +6543,16 @@
         <v>1</v>
       </c>
       <c r="G191" t="n">
-        <v>202.6999969482422</v>
+        <v>20270</v>
       </c>
       <c r="H191" t="n">
-        <v>202.3999938964844</v>
+        <v>20240</v>
       </c>
       <c r="I191" t="n">
-        <v>405.0999908447266</v>
+        <v>40510</v>
       </c>
       <c r="J191" t="n">
-        <v>1.001482228561288</v>
+        <v>1.001482213438735</v>
       </c>
       <c r="K191" s="1" t="n">
         <v>46100.625</v>
@@ -6577,10 +6577,10 @@
       </c>
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="n">
-        <v>205.3999938964844</v>
+        <v>20540</v>
       </c>
       <c r="I192" t="n">
-        <v>205.3999938964844</v>
+        <v>20540</v>
       </c>
       <c r="J192" t="inlineStr"/>
       <c r="K192" s="1" t="n">
@@ -6607,16 +6607,16 @@
         <v>1</v>
       </c>
       <c r="G193" t="n">
-        <v>213.1999969482422</v>
+        <v>21320</v>
       </c>
       <c r="H193" t="n">
-        <v>205.3999938964844</v>
+        <v>20540</v>
       </c>
       <c r="I193" t="n">
-        <v>418.5999908447266</v>
+        <v>41860</v>
       </c>
       <c r="J193" t="n">
-        <v>1.037974699530365</v>
+        <v>1.037974683544304</v>
       </c>
       <c r="K193" s="1" t="n">
         <v>46100.625</v>
@@ -6641,10 +6641,10 @@
       </c>
       <c r="G194" t="inlineStr"/>
       <c r="H194" t="n">
-        <v>202</v>
+        <v>20200</v>
       </c>
       <c r="I194" t="n">
-        <v>202</v>
+        <v>20200</v>
       </c>
       <c r="J194" t="inlineStr"/>
       <c r="K194" s="1" t="n">
@@ -6671,16 +6671,16 @@
         <v>1</v>
       </c>
       <c r="G195" t="n">
-        <v>217.1999969482422</v>
+        <v>21720</v>
       </c>
       <c r="H195" t="n">
-        <v>202</v>
+        <v>20200</v>
       </c>
       <c r="I195" t="n">
-        <v>419.1999969482422</v>
+        <v>41920</v>
       </c>
       <c r="J195" t="n">
-        <v>1.075247509644763</v>
+        <v>1.075247524752475</v>
       </c>
       <c r="K195" s="1" t="n">
         <v>46100.625</v>
@@ -6705,10 +6705,10 @@
       </c>
       <c r="G196" t="inlineStr"/>
       <c r="H196" t="n">
-        <v>199.6000061035156</v>
+        <v>19960</v>
       </c>
       <c r="I196" t="n">
-        <v>199.6000061035156</v>
+        <v>19960</v>
       </c>
       <c r="J196" t="inlineStr"/>
       <c r="K196" s="1" t="n">
@@ -6735,16 +6735,16 @@
         <v>1</v>
       </c>
       <c r="G197" t="n">
-        <v>213.6999969482422</v>
+        <v>21370</v>
       </c>
       <c r="H197" t="n">
-        <v>199.6000061035156</v>
+        <v>19960</v>
       </c>
       <c r="I197" t="n">
-        <v>413.3000030517578</v>
+        <v>41330</v>
       </c>
       <c r="J197" t="n">
-        <v>1.070641234536907</v>
+        <v>1.07064128256513</v>
       </c>
       <c r="K197" s="1" t="n">
         <v>46100.625</v>
@@ -6769,10 +6769,10 @@
       </c>
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="n">
-        <v>196.6000061035156</v>
+        <v>19660</v>
       </c>
       <c r="I198" t="n">
-        <v>196.6000061035156</v>
+        <v>19660</v>
       </c>
       <c r="J198" t="inlineStr"/>
       <c r="K198" s="1" t="n">
@@ -6799,16 +6799,16 @@
         <v>1</v>
       </c>
       <c r="G199" t="n">
-        <v>207.8999938964844</v>
+        <v>20790</v>
       </c>
       <c r="H199" t="n">
-        <v>196.6000061035156</v>
+        <v>19660</v>
       </c>
       <c r="I199" t="n">
-        <v>404.5</v>
+        <v>40450</v>
       </c>
       <c r="J199" t="n">
-        <v>1.057477047009953</v>
+        <v>1.057477110885046</v>
       </c>
       <c r="K199" s="1" t="n">
         <v>46100.625</v>
@@ -6833,10 +6833,10 @@
       </c>
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="n">
-        <v>181.6000061035156</v>
+        <v>18160</v>
       </c>
       <c r="I200" t="n">
-        <v>181.6000061035156</v>
+        <v>18160</v>
       </c>
       <c r="J200" t="inlineStr"/>
       <c r="K200" s="1" t="n">
@@ -6863,16 +6863,16 @@
         <v>1</v>
       </c>
       <c r="G201" t="n">
-        <v>197.1000061035156</v>
+        <v>19710</v>
       </c>
       <c r="H201" t="n">
-        <v>181.6000061035156</v>
+        <v>18160</v>
       </c>
       <c r="I201" t="n">
-        <v>378.7000122070312</v>
+        <v>37870</v>
       </c>
       <c r="J201" t="n">
-        <v>1.085352420038822</v>
+        <v>1.085352422907489</v>
       </c>
       <c r="K201" s="1" t="n">
         <v>46100.625</v>
@@ -6897,10 +6897,10 @@
       </c>
       <c r="G202" t="inlineStr"/>
       <c r="H202" t="n">
-        <v>167.3000030517578</v>
+        <v>16730</v>
       </c>
       <c r="I202" t="n">
-        <v>167.3000030517578</v>
+        <v>16730</v>
       </c>
       <c r="J202" t="inlineStr"/>
       <c r="K202" s="1" t="n">
@@ -6927,16 +6927,16 @@
         <v>1</v>
       </c>
       <c r="G203" t="n">
-        <v>185</v>
+        <v>18500</v>
       </c>
       <c r="H203" t="n">
-        <v>167.3000030517578</v>
+        <v>16730</v>
       </c>
       <c r="I203" t="n">
-        <v>352.3000030517578</v>
+        <v>35230</v>
       </c>
       <c r="J203" t="n">
-        <v>1.105797947551539</v>
+        <v>1.105797967722654</v>
       </c>
       <c r="K203" s="1" t="n">
         <v>46100.625</v>
@@ -6961,10 +6961,10 @@
       </c>
       <c r="G204" t="inlineStr"/>
       <c r="H204" t="n">
-        <v>159.8999938964844</v>
+        <v>15990</v>
       </c>
       <c r="I204" t="n">
-        <v>159.8999938964844</v>
+        <v>15990</v>
       </c>
       <c r="J204" t="inlineStr"/>
       <c r="K204" s="1" t="n">
@@ -6991,16 +6991,16 @@
         <v>1</v>
       </c>
       <c r="G205" t="n">
-        <v>183.6000061035156</v>
+        <v>18360</v>
       </c>
       <c r="H205" t="n">
-        <v>159.8999938964844</v>
+        <v>15990</v>
       </c>
       <c r="I205" t="n">
-        <v>343.5</v>
+        <v>34350</v>
       </c>
       <c r="J205" t="n">
-        <v>1.148217718021766</v>
+        <v>1.148217636022514</v>
       </c>
       <c r="K205" s="1" t="n">
         <v>46100.625</v>
@@ -7025,10 +7025,10 @@
       </c>
       <c r="G206" t="inlineStr"/>
       <c r="H206" t="n">
-        <v>157.5</v>
+        <v>15750</v>
       </c>
       <c r="I206" t="n">
-        <v>157.5</v>
+        <v>15750</v>
       </c>
       <c r="J206" t="inlineStr"/>
       <c r="K206" s="1" t="n">
@@ -7055,16 +7055,16 @@
         <v>1</v>
       </c>
       <c r="G207" t="n">
-        <v>195.8000030517578</v>
+        <v>19580</v>
       </c>
       <c r="H207" t="n">
-        <v>157.5</v>
+        <v>15750</v>
       </c>
       <c r="I207" t="n">
-        <v>353.3000030517578</v>
+        <v>35330</v>
       </c>
       <c r="J207" t="n">
-        <v>1.243174622550843</v>
+        <v>1.243174603174603</v>
       </c>
       <c r="K207" s="1" t="n">
         <v>46100.625</v>
@@ -7089,10 +7089,10 @@
       </c>
       <c r="G208" t="inlineStr"/>
       <c r="H208" t="n">
-        <v>156.8000030517578</v>
+        <v>15680</v>
       </c>
       <c r="I208" t="n">
-        <v>156.8000030517578</v>
+        <v>15680</v>
       </c>
       <c r="J208" t="inlineStr"/>
       <c r="K208" s="1" t="n">
@@ -7119,16 +7119,16 @@
         <v>1</v>
       </c>
       <c r="G209" t="n">
-        <v>207.1999969482422</v>
+        <v>20720</v>
       </c>
       <c r="H209" t="n">
-        <v>156.8000030517578</v>
+        <v>15680</v>
       </c>
       <c r="I209" t="n">
-        <v>364</v>
+        <v>36400</v>
       </c>
       <c r="J209" t="n">
-        <v>1.321428526247209</v>
+        <v>1.321428571428571</v>
       </c>
       <c r="K209" s="1" t="n">
         <v>46100.625</v>
@@ -7153,10 +7153,10 @@
       </c>
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="n">
-        <v>156.3999938964844</v>
+        <v>15640</v>
       </c>
       <c r="I210" t="n">
-        <v>156.3999938964844</v>
+        <v>15640</v>
       </c>
       <c r="J210" t="inlineStr"/>
       <c r="K210" s="1" t="n">
@@ -7183,16 +7183,16 @@
         <v>1</v>
       </c>
       <c r="G211" t="n">
-        <v>217.1999969482422</v>
+        <v>21720</v>
       </c>
       <c r="H211" t="n">
-        <v>156.3999938964844</v>
+        <v>15640</v>
       </c>
       <c r="I211" t="n">
-        <v>373.5999908447266</v>
+        <v>37360</v>
       </c>
       <c r="J211" t="n">
-        <v>1.388746837752431</v>
+        <v>1.388746803069054</v>
       </c>
       <c r="K211" s="1" t="n">
         <v>46100.625</v>
@@ -7217,10 +7217,10 @@
       </c>
       <c r="G212" t="inlineStr"/>
       <c r="H212" t="n">
-        <v>160.3999938964844</v>
+        <v>16040</v>
       </c>
       <c r="I212" t="n">
-        <v>160.3999938964844</v>
+        <v>16040</v>
       </c>
       <c r="J212" t="inlineStr"/>
       <c r="K212" s="1" t="n">
@@ -7247,16 +7247,16 @@
         <v>1</v>
       </c>
       <c r="G213" t="n">
-        <v>242.6999969482422</v>
+        <v>24270</v>
       </c>
       <c r="H213" t="n">
-        <v>160.3999938964844</v>
+        <v>16040</v>
       </c>
       <c r="I213" t="n">
-        <v>403.0999908447266</v>
+        <v>40310</v>
       </c>
       <c r="J213" t="n">
-        <v>1.513092307876713</v>
+        <v>1.513092269326683</v>
       </c>
       <c r="K213" s="1" t="n">
         <v>46100.625</v>
@@ -7281,10 +7281,10 @@
       </c>
       <c r="G214" t="inlineStr"/>
       <c r="H214" t="n">
-        <v>180.6000061035156</v>
+        <v>18060</v>
       </c>
       <c r="I214" t="n">
-        <v>180.6000061035156</v>
+        <v>18060</v>
       </c>
       <c r="J214" t="inlineStr"/>
       <c r="K214" s="1" t="n">
@@ -7311,16 +7311,16 @@
         <v>1</v>
       </c>
       <c r="G215" t="n">
-        <v>276.6000061035156</v>
+        <v>27660</v>
       </c>
       <c r="H215" t="n">
-        <v>180.6000061035156</v>
+        <v>18060</v>
       </c>
       <c r="I215" t="n">
-        <v>457.2000122070312</v>
+        <v>45720</v>
       </c>
       <c r="J215" t="n">
-        <v>1.531561443829493</v>
+        <v>1.53156146179402</v>
       </c>
       <c r="K215" s="1" t="n">
         <v>46100.625</v>
@@ -7345,10 +7345,10 @@
       </c>
       <c r="G216" t="inlineStr"/>
       <c r="H216" t="n">
-        <v>215.5</v>
+        <v>21550</v>
       </c>
       <c r="I216" t="n">
-        <v>215.5</v>
+        <v>21550</v>
       </c>
       <c r="J216" t="inlineStr"/>
       <c r="K216" s="1" t="n">
@@ -7375,16 +7375,16 @@
         <v>1</v>
       </c>
       <c r="G217" t="n">
-        <v>290.2000122070312</v>
+        <v>29020</v>
       </c>
       <c r="H217" t="n">
-        <v>215.5</v>
+        <v>21550</v>
       </c>
       <c r="I217" t="n">
-        <v>505.7000122070312</v>
+        <v>50570</v>
       </c>
       <c r="J217" t="n">
-        <v>1.346635787503625</v>
+        <v>1.346635730858469</v>
       </c>
       <c r="K217" s="1" t="n">
         <v>46100.625</v>
@@ -7409,10 +7409,10 @@
       </c>
       <c r="G218" t="inlineStr"/>
       <c r="H218" t="n">
-        <v>236.3000030517578</v>
+        <v>23630</v>
       </c>
       <c r="I218" t="n">
-        <v>236.3000030517578</v>
+        <v>23630</v>
       </c>
       <c r="J218" t="inlineStr"/>
       <c r="K218" s="1" t="n">
@@ -7439,16 +7439,16 @@
         <v>1</v>
       </c>
       <c r="G219" t="n">
-        <v>280.7999877929688</v>
+        <v>28080</v>
       </c>
       <c r="H219" t="n">
-        <v>236.3000030517578</v>
+        <v>23630</v>
       </c>
       <c r="I219" t="n">
-        <v>517.0999908447266</v>
+        <v>51710</v>
       </c>
       <c r="J219" t="n">
-        <v>1.188319865283556</v>
+        <v>1.188319932289463</v>
       </c>
       <c r="K219" s="1" t="n">
         <v>46100.625</v>
@@ -7473,10 +7473,10 @@
       </c>
       <c r="G220" t="inlineStr"/>
       <c r="H220" t="n">
-        <v>241.8000030517578</v>
+        <v>24180</v>
       </c>
       <c r="I220" t="n">
-        <v>241.8000030517578</v>
+        <v>24180</v>
       </c>
       <c r="J220" t="inlineStr"/>
       <c r="K220" s="1" t="n">
@@ -7503,16 +7503,16 @@
         <v>1</v>
       </c>
       <c r="G221" t="n">
-        <v>270.7000122070312</v>
+        <v>27070</v>
       </c>
       <c r="H221" t="n">
-        <v>241.8000030517578</v>
+        <v>24180</v>
       </c>
       <c r="I221" t="n">
-        <v>512.5000152587891</v>
+        <v>51250</v>
       </c>
       <c r="J221" t="n">
-        <v>1.119520301036089</v>
+        <v>1.119520264681555</v>
       </c>
       <c r="K221" s="1" t="n">
         <v>46100.625</v>
@@ -7537,10 +7537,10 @@
       </c>
       <c r="G222" t="inlineStr"/>
       <c r="H222" t="n">
-        <v>249.6000061035156</v>
+        <v>24960</v>
       </c>
       <c r="I222" t="n">
-        <v>249.6000061035156</v>
+        <v>24960</v>
       </c>
       <c r="J222" t="inlineStr"/>
       <c r="K222" s="1" t="n">
@@ -7567,16 +7567,16 @@
         <v>1</v>
       </c>
       <c r="G223" t="n">
-        <v>264.7999877929688</v>
+        <v>26480</v>
       </c>
       <c r="H223" t="n">
-        <v>249.6000061035156</v>
+        <v>24960</v>
       </c>
       <c r="I223" t="n">
-        <v>514.3999938964844</v>
+        <v>51440</v>
       </c>
       <c r="J223" t="n">
-        <v>1.060897361048738</v>
+        <v>1.060897435897436</v>
       </c>
       <c r="K223" s="1" t="n">
         <v>46100.625</v>
@@ -7601,10 +7601,10 @@
       </c>
       <c r="G224" t="inlineStr"/>
       <c r="H224" t="n">
-        <v>256.2999877929688</v>
+        <v>25630</v>
       </c>
       <c r="I224" t="n">
-        <v>256.2999877929688</v>
+        <v>25630</v>
       </c>
       <c r="J224" t="inlineStr"/>
       <c r="K224" s="1" t="n">
@@ -7631,16 +7631,16 @@
         <v>1</v>
       </c>
       <c r="G225" t="n">
-        <v>264.3999938964844</v>
+        <v>26440</v>
       </c>
       <c r="H225" t="n">
-        <v>256.2999877929688</v>
+        <v>25630</v>
       </c>
       <c r="I225" t="n">
-        <v>520.6999816894531</v>
+        <v>52070</v>
       </c>
       <c r="J225" t="n">
-        <v>1.031603614862669</v>
+        <v>1.031603589543504</v>
       </c>
       <c r="K225" s="1" t="n">
         <v>46100.625</v>
@@ -7665,10 +7665,10 @@
       </c>
       <c r="G226" t="inlineStr"/>
       <c r="H226" t="n">
-        <v>254.8999938964844</v>
+        <v>25490</v>
       </c>
       <c r="I226" t="n">
-        <v>254.8999938964844</v>
+        <v>25490</v>
       </c>
       <c r="J226" t="inlineStr"/>
       <c r="K226" s="1" t="n">
@@ -7695,16 +7695,16 @@
         <v>1</v>
       </c>
       <c r="G227" t="n">
-        <v>261.6000061035156</v>
+        <v>26160</v>
       </c>
       <c r="H227" t="n">
-        <v>254.8999938964844</v>
+        <v>25490</v>
       </c>
       <c r="I227" t="n">
-        <v>516.5</v>
+        <v>51650</v>
       </c>
       <c r="J227" t="n">
-        <v>1.026284866094395</v>
+        <v>1.02628481757552</v>
       </c>
       <c r="K227" s="1" t="n">
         <v>46100.625</v>
@@ -7729,10 +7729,10 @@
       </c>
       <c r="G228" t="inlineStr"/>
       <c r="H228" t="n">
-        <v>239.3999938964844</v>
+        <v>23940</v>
       </c>
       <c r="I228" t="n">
-        <v>239.3999938964844</v>
+        <v>23940</v>
       </c>
       <c r="J228" t="inlineStr"/>
       <c r="K228" s="1" t="n">
@@ -7759,16 +7759,16 @@
         <v>1</v>
       </c>
       <c r="G229" t="n">
-        <v>254.3000030517578</v>
+        <v>25430</v>
       </c>
       <c r="H229" t="n">
-        <v>239.3999938964844</v>
+        <v>23940</v>
       </c>
       <c r="I229" t="n">
-        <v>493.6999969482422</v>
+        <v>49370</v>
       </c>
       <c r="J229" t="n">
-        <v>1.062238970489348</v>
+        <v>1.062238930659983</v>
       </c>
       <c r="K229" s="1" t="n">
         <v>46100.625</v>
@@ -7793,10 +7793,10 @@
       </c>
       <c r="G230" t="inlineStr"/>
       <c r="H230" t="n">
-        <v>218.5</v>
+        <v>21850</v>
       </c>
       <c r="I230" t="n">
-        <v>218.5</v>
+        <v>21850</v>
       </c>
       <c r="J230" t="inlineStr"/>
       <c r="K230" s="1" t="n">
@@ -7823,16 +7823,16 @@
         <v>1</v>
       </c>
       <c r="G231" t="n">
-        <v>258.2000122070312</v>
+        <v>25820</v>
       </c>
       <c r="H231" t="n">
-        <v>218.5</v>
+        <v>21850</v>
       </c>
       <c r="I231" t="n">
-        <v>476.7000122070312</v>
+        <v>47670</v>
       </c>
       <c r="J231" t="n">
-        <v>1.181693419711813</v>
+        <v>1.181693363844394</v>
       </c>
       <c r="K231" s="1" t="n">
         <v>46100.625</v>
@@ -7857,10 +7857,10 @@
       </c>
       <c r="G232" t="inlineStr"/>
       <c r="H232" t="n">
-        <v>222.3999938964844</v>
+        <v>22240</v>
       </c>
       <c r="I232" t="n">
-        <v>222.3999938964844</v>
+        <v>22240</v>
       </c>
       <c r="J232" t="inlineStr"/>
       <c r="K232" s="1" t="n">
@@ -7887,16 +7887,16 @@
         <v>1</v>
       </c>
       <c r="G233" t="n">
-        <v>269.7999877929688</v>
+        <v>26980</v>
       </c>
       <c r="H233" t="n">
-        <v>222.3999938964844</v>
+        <v>22240</v>
       </c>
       <c r="I233" t="n">
-        <v>492.1999816894531</v>
+        <v>49220</v>
       </c>
       <c r="J233" t="n">
-        <v>1.213129474808109</v>
+        <v>1.213129496402878</v>
       </c>
       <c r="K233" s="1" t="n">
         <v>46100.625</v>
@@ -7921,10 +7921,10 @@
       </c>
       <c r="G234" t="inlineStr"/>
       <c r="H234" t="n">
-        <v>245.6999969482422</v>
+        <v>24570</v>
       </c>
       <c r="I234" t="n">
-        <v>245.6999969482422</v>
+        <v>24570</v>
       </c>
       <c r="J234" t="inlineStr"/>
       <c r="K234" s="1" t="n">
@@ -7951,16 +7951,16 @@
         <v>1</v>
       </c>
       <c r="G235" t="n">
-        <v>269.3999938964844</v>
+        <v>26940</v>
       </c>
       <c r="H235" t="n">
-        <v>245.6999969482422</v>
+        <v>24570</v>
       </c>
       <c r="I235" t="n">
-        <v>515.0999908447266</v>
+        <v>51510</v>
       </c>
       <c r="J235" t="n">
-        <v>1.096459085236516</v>
+        <v>1.096459096459097</v>
       </c>
       <c r="K235" s="1" t="n">
         <v>46100.625</v>
@@ -7985,10 +7985,10 @@
       </c>
       <c r="G236" t="inlineStr"/>
       <c r="H236" t="n">
-        <v>260</v>
+        <v>26000</v>
       </c>
       <c r="I236" t="n">
-        <v>260</v>
+        <v>26000</v>
       </c>
       <c r="J236" t="inlineStr"/>
       <c r="K236" s="1" t="n">
@@ -8015,16 +8015,16 @@
         <v>1</v>
       </c>
       <c r="G237" t="n">
-        <v>259.2999877929688</v>
+        <v>25930</v>
       </c>
       <c r="H237" t="n">
-        <v>260</v>
+        <v>26000</v>
       </c>
       <c r="I237" t="n">
-        <v>519.2999877929688</v>
+        <v>51930</v>
       </c>
       <c r="J237" t="n">
-        <v>0.9973076453575721</v>
+        <v>0.9973076923076923</v>
       </c>
       <c r="K237" s="1" t="n">
         <v>46100.625</v>
@@ -8049,10 +8049,10 @@
       </c>
       <c r="G238" t="inlineStr"/>
       <c r="H238" t="n">
-        <v>279.5</v>
+        <v>27950</v>
       </c>
       <c r="I238" t="n">
-        <v>279.5</v>
+        <v>27950</v>
       </c>
       <c r="J238" t="inlineStr"/>
       <c r="K238" s="1" t="n">
@@ -8079,16 +8079,16 @@
         <v>1</v>
       </c>
       <c r="G239" t="n">
-        <v>255.6000061035156</v>
+        <v>25560</v>
       </c>
       <c r="H239" t="n">
-        <v>279.5</v>
+        <v>27950</v>
       </c>
       <c r="I239" t="n">
-        <v>535.1000061035156</v>
+        <v>53510</v>
       </c>
       <c r="J239" t="n">
-        <v>0.9144901828390541</v>
+        <v>0.9144901610017889</v>
       </c>
       <c r="K239" s="1" t="n">
         <v>46100.625</v>
@@ -8113,10 +8113,10 @@
       </c>
       <c r="G240" t="inlineStr"/>
       <c r="H240" t="n">
-        <v>298.1000061035156</v>
+        <v>29810</v>
       </c>
       <c r="I240" t="n">
-        <v>298.1000061035156</v>
+        <v>29810</v>
       </c>
       <c r="J240" t="inlineStr"/>
       <c r="K240" s="1" t="n">
@@ -8143,16 +8143,16 @@
         <v>1</v>
       </c>
       <c r="G241" t="n">
-        <v>259.3999938964844</v>
+        <v>25940</v>
       </c>
       <c r="H241" t="n">
-        <v>298.1000061035156</v>
+        <v>29810</v>
       </c>
       <c r="I241" t="n">
-        <v>557.5</v>
+        <v>55750</v>
       </c>
       <c r="J241" t="n">
-        <v>0.8701777543956419</v>
+        <v>0.8701777926870178</v>
       </c>
       <c r="K241" s="1" t="n">
         <v>46100.625</v>
@@ -8177,10 +8177,10 @@
       </c>
       <c r="G242" t="inlineStr"/>
       <c r="H242" t="n">
-        <v>289.5</v>
+        <v>28950</v>
       </c>
       <c r="I242" t="n">
-        <v>289.5</v>
+        <v>28950</v>
       </c>
       <c r="J242" t="inlineStr"/>
       <c r="K242" s="1" t="n">
@@ -8207,16 +8207,16 @@
         <v>1</v>
       </c>
       <c r="G243" t="n">
-        <v>268.8999938964844</v>
+        <v>26890</v>
       </c>
       <c r="H243" t="n">
-        <v>289.5</v>
+        <v>28950</v>
       </c>
       <c r="I243" t="n">
-        <v>558.3999938964844</v>
+        <v>55840</v>
       </c>
       <c r="J243" t="n">
-        <v>0.9288428113868199</v>
+        <v>0.9288428324697755</v>
       </c>
       <c r="K243" s="1" t="n">
         <v>46100.625</v>
@@ -8241,10 +8241,10 @@
       </c>
       <c r="G244" t="inlineStr"/>
       <c r="H244" t="n">
-        <v>262.8999938964844</v>
+        <v>26290</v>
       </c>
       <c r="I244" t="n">
-        <v>262.8999938964844</v>
+        <v>26290</v>
       </c>
       <c r="J244" t="inlineStr"/>
       <c r="K244" s="1" t="n">
@@ -8271,16 +8271,16 @@
         <v>1</v>
       </c>
       <c r="G245" t="n">
-        <v>277.7000122070312</v>
+        <v>27770</v>
       </c>
       <c r="H245" t="n">
-        <v>262.8999938964844</v>
+        <v>26290</v>
       </c>
       <c r="I245" t="n">
-        <v>540.6000061035156</v>
+        <v>54060</v>
       </c>
       <c r="J245" t="n">
-        <v>1.056295240221171</v>
+        <v>1.056295169265881</v>
       </c>
       <c r="K245" s="1" t="n">
         <v>46100.625</v>
@@ -8305,10 +8305,10 @@
       </c>
       <c r="G246" t="inlineStr"/>
       <c r="H246" t="n">
-        <v>221.3999938964844</v>
+        <v>22140</v>
       </c>
       <c r="I246" t="n">
-        <v>221.3999938964844</v>
+        <v>22140</v>
       </c>
       <c r="J246" t="inlineStr"/>
       <c r="K246" s="1" t="n">
@@ -8335,16 +8335,16 @@
         <v>1</v>
       </c>
       <c r="G247" t="n">
-        <v>266.3999938964844</v>
+        <v>26640</v>
       </c>
       <c r="H247" t="n">
-        <v>221.3999938964844</v>
+        <v>22140</v>
       </c>
       <c r="I247" t="n">
-        <v>487.7999877929688</v>
+        <v>48780</v>
       </c>
       <c r="J247" t="n">
-        <v>1.203252038123541</v>
+        <v>1.203252032520325</v>
       </c>
       <c r="K247" s="1" t="n">
         <v>46100.625</v>
@@ -8369,10 +8369,10 @@
       </c>
       <c r="G248" t="inlineStr"/>
       <c r="H248" t="n">
-        <v>187.3999938964844</v>
+        <v>18740</v>
       </c>
       <c r="I248" t="n">
-        <v>187.3999938964844</v>
+        <v>18740</v>
       </c>
       <c r="J248" t="inlineStr"/>
       <c r="K248" s="1" t="n">
@@ -8399,16 +8399,16 @@
         <v>1</v>
       </c>
       <c r="G249" t="n">
-        <v>252.8999938964844</v>
+        <v>25290</v>
       </c>
       <c r="H249" t="n">
-        <v>187.3999938964844</v>
+        <v>18740</v>
       </c>
       <c r="I249" t="n">
-        <v>440.2999877929688</v>
+        <v>44030</v>
       </c>
       <c r="J249" t="n">
-        <v>1.349519755247061</v>
+        <v>1.349519743863394</v>
       </c>
       <c r="K249" s="1" t="n">
         <v>46100.625</v>
@@ -8433,10 +8433,10 @@
       </c>
       <c r="G250" t="inlineStr"/>
       <c r="H250" t="n">
-        <v>186.1999969482422</v>
+        <v>18620</v>
       </c>
       <c r="I250" t="n">
-        <v>186.1999969482422</v>
+        <v>18620</v>
       </c>
       <c r="J250" t="inlineStr"/>
       <c r="K250" s="1" t="n">
@@ -8463,16 +8463,16 @@
         <v>1</v>
       </c>
       <c r="G251" t="n">
-        <v>250.3999938964844</v>
+        <v>25040</v>
       </c>
       <c r="H251" t="n">
-        <v>186.1999969482422</v>
+        <v>18620</v>
       </c>
       <c r="I251" t="n">
-        <v>436.5999908447266</v>
+        <v>43660</v>
       </c>
       <c r="J251" t="n">
-        <v>1.344790537059395</v>
+        <v>1.344790547798067</v>
       </c>
       <c r="K251" s="1" t="n">
         <v>46100.625</v>
@@ -8497,10 +8497,10 @@
       </c>
       <c r="G252" t="inlineStr"/>
       <c r="H252" t="n">
-        <v>195.3999938964844</v>
+        <v>19540</v>
       </c>
       <c r="I252" t="n">
-        <v>195.3999938964844</v>
+        <v>19540</v>
       </c>
       <c r="J252" t="inlineStr"/>
       <c r="K252" s="1" t="n">
@@ -8527,16 +8527,16 @@
         <v>1</v>
       </c>
       <c r="G253" t="n">
-        <v>245.8000030517578</v>
+        <v>24580</v>
       </c>
       <c r="H253" t="n">
-        <v>195.3999938964844</v>
+        <v>19540</v>
       </c>
       <c r="I253" t="n">
-        <v>441.1999969482422</v>
+        <v>44120</v>
       </c>
       <c r="J253" t="n">
-        <v>1.257932501174864</v>
+        <v>1.257932446264074</v>
       </c>
       <c r="K253" s="1" t="n">
         <v>46100.625</v>
@@ -8561,10 +8561,10 @@
       </c>
       <c r="G254" t="inlineStr"/>
       <c r="H254" t="n">
-        <v>194.1000061035156</v>
+        <v>19410</v>
       </c>
       <c r="I254" t="n">
-        <v>194.1000061035156</v>
+        <v>19410</v>
       </c>
       <c r="J254" t="inlineStr"/>
       <c r="K254" s="1" t="n">
@@ -8591,16 +8591,16 @@
         <v>1</v>
       </c>
       <c r="G255" t="n">
-        <v>237.6999969482422</v>
+        <v>23770</v>
       </c>
       <c r="H255" t="n">
-        <v>194.1000061035156</v>
+        <v>19410</v>
       </c>
       <c r="I255" t="n">
-        <v>431.8000030517578</v>
+        <v>43180</v>
       </c>
       <c r="J255" t="n">
-        <v>1.224626426964017</v>
+        <v>1.22462648119526</v>
       </c>
       <c r="K255" s="1" t="n">
         <v>46100.625</v>
@@ -8625,10 +8625,10 @@
       </c>
       <c r="G256" t="inlineStr"/>
       <c r="H256" t="n">
-        <v>189.6000061035156</v>
+        <v>18960</v>
       </c>
       <c r="I256" t="n">
-        <v>189.6000061035156</v>
+        <v>18960</v>
       </c>
       <c r="J256" t="inlineStr"/>
       <c r="K256" s="1" t="n">
@@ -8655,16 +8655,16 @@
         <v>1</v>
       </c>
       <c r="G257" t="n">
-        <v>225.3999938964844</v>
+        <v>22540</v>
       </c>
       <c r="H257" t="n">
-        <v>189.6000061035156</v>
+        <v>18960</v>
       </c>
       <c r="I257" t="n">
-        <v>415</v>
+        <v>41500</v>
       </c>
       <c r="J257" t="n">
-        <v>1.18881849493941</v>
+        <v>1.188818565400844</v>
       </c>
       <c r="K257" s="1" t="n">
         <v>46100.625</v>
@@ -8689,10 +8689,10 @@
       </c>
       <c r="G258" t="inlineStr"/>
       <c r="H258" t="n">
-        <v>187.3999938964844</v>
+        <v>18740</v>
       </c>
       <c r="I258" t="n">
-        <v>187.3999938964844</v>
+        <v>18740</v>
       </c>
       <c r="J258" t="inlineStr"/>
       <c r="K258" s="1" t="n">
@@ -8719,16 +8719,16 @@
         <v>1</v>
       </c>
       <c r="G259" t="n">
-        <v>215.6999969482422</v>
+        <v>21570</v>
       </c>
       <c r="H259" t="n">
-        <v>187.3999938964844</v>
+        <v>18740</v>
       </c>
       <c r="I259" t="n">
-        <v>403.0999908447266</v>
+        <v>40310</v>
       </c>
       <c r="J259" t="n">
-        <v>1.151013895269336</v>
+        <v>1.151013874066169</v>
       </c>
       <c r="K259" s="1" t="n">
         <v>46100.625</v>
@@ -8753,10 +8753,10 @@
       </c>
       <c r="G260" t="inlineStr"/>
       <c r="H260" t="n">
-        <v>189.8000030517578</v>
+        <v>18980</v>
       </c>
       <c r="I260" t="n">
-        <v>189.8000030517578</v>
+        <v>18980</v>
       </c>
       <c r="J260" t="inlineStr"/>
       <c r="K260" s="1" t="n">
@@ -8783,16 +8783,16 @@
         <v>1</v>
       </c>
       <c r="G261" t="n">
-        <v>205.5</v>
+        <v>20550</v>
       </c>
       <c r="H261" t="n">
-        <v>189.8000030517578</v>
+        <v>18980</v>
       </c>
       <c r="I261" t="n">
-        <v>395.3000030517578</v>
+        <v>39530</v>
       </c>
       <c r="J261" t="n">
-        <v>1.082718633802977</v>
+        <v>1.082718651211802</v>
       </c>
       <c r="K261" s="1" t="n">
         <v>46100.625</v>
@@ -8817,10 +8817,10 @@
       </c>
       <c r="G262" t="inlineStr"/>
       <c r="H262" t="n">
-        <v>198.1000061035156</v>
+        <v>19810</v>
       </c>
       <c r="I262" t="n">
-        <v>198.1000061035156</v>
+        <v>19810</v>
       </c>
       <c r="J262" t="inlineStr"/>
       <c r="K262" s="1" t="n">
@@ -8847,16 +8847,16 @@
         <v>1</v>
       </c>
       <c r="G263" t="n">
-        <v>196.3000030517578</v>
+        <v>19630</v>
       </c>
       <c r="H263" t="n">
-        <v>198.1000061035156</v>
+        <v>19810</v>
       </c>
       <c r="I263" t="n">
-        <v>394.4000091552734</v>
+        <v>39440</v>
       </c>
       <c r="J263" t="n">
-        <v>0.990913664834431</v>
+        <v>0.9909136799596163</v>
       </c>
       <c r="K263" s="1" t="n">
         <v>46100.625</v>
@@ -8881,10 +8881,10 @@
       </c>
       <c r="G264" t="inlineStr"/>
       <c r="H264" t="n">
-        <v>202.1999969482422</v>
+        <v>20220</v>
       </c>
       <c r="I264" t="n">
-        <v>202.1999969482422</v>
+        <v>20220</v>
       </c>
       <c r="J264" t="inlineStr"/>
       <c r="K264" s="1" t="n">
@@ -8911,16 +8911,16 @@
         <v>1</v>
       </c>
       <c r="G265" t="n">
-        <v>196.8000030517578</v>
+        <v>19680</v>
       </c>
       <c r="H265" t="n">
-        <v>202.1999969482422</v>
+        <v>20220</v>
       </c>
       <c r="I265" t="n">
-        <v>399</v>
+        <v>39900</v>
       </c>
       <c r="J265" t="n">
-        <v>0.9732937983284607</v>
+        <v>0.973293768545994</v>
       </c>
       <c r="K265" s="1" t="n">
         <v>46100.625</v>
@@ -8945,10 +8945,10 @@
       </c>
       <c r="G266" t="inlineStr"/>
       <c r="H266" t="n">
-        <v>200.5</v>
+        <v>20050</v>
       </c>
       <c r="I266" t="n">
-        <v>200.5</v>
+        <v>20050</v>
       </c>
       <c r="J266" t="inlineStr"/>
       <c r="K266" s="1" t="n">
@@ -8975,16 +8975,16 @@
         <v>1</v>
       </c>
       <c r="G267" t="n">
-        <v>197.8000030517578</v>
+        <v>19780</v>
       </c>
       <c r="H267" t="n">
-        <v>200.5</v>
+        <v>20050</v>
       </c>
       <c r="I267" t="n">
-        <v>398.3000030517578</v>
+        <v>39830</v>
       </c>
       <c r="J267" t="n">
-        <v>0.9865336810561487</v>
+        <v>0.9865336658354115</v>
       </c>
       <c r="K267" s="1" t="n">
         <v>46100.625</v>
@@ -9009,10 +9009,10 @@
       </c>
       <c r="G268" t="inlineStr"/>
       <c r="H268" t="n">
-        <v>196.1999969482422</v>
+        <v>19620</v>
       </c>
       <c r="I268" t="n">
-        <v>196.1999969482422</v>
+        <v>19620</v>
       </c>
       <c r="J268" t="inlineStr"/>
       <c r="K268" s="1" t="n">
@@ -9039,16 +9039,16 @@
         <v>1</v>
       </c>
       <c r="G269" t="n">
-        <v>195.8999938964844</v>
+        <v>19590</v>
       </c>
       <c r="H269" t="n">
-        <v>196.1999969482422</v>
+        <v>19620</v>
       </c>
       <c r="I269" t="n">
-        <v>392.0999908447266</v>
+        <v>39210</v>
       </c>
       <c r="J269" t="n">
-        <v>0.9984709324341277</v>
+        <v>0.9984709480122325</v>
       </c>
       <c r="K269" s="1" t="n">
         <v>46100.625</v>
@@ -9073,10 +9073,10 @@
       </c>
       <c r="G270" t="inlineStr"/>
       <c r="H270" t="n">
-        <v>197.5</v>
+        <v>19750</v>
       </c>
       <c r="I270" t="n">
-        <v>197.5</v>
+        <v>19750</v>
       </c>
       <c r="J270" t="inlineStr"/>
       <c r="K270" s="1" t="n">
@@ -9103,16 +9103,16 @@
         <v>1</v>
       </c>
       <c r="G271" t="n">
-        <v>198.1000061035156</v>
+        <v>19810</v>
       </c>
       <c r="H271" t="n">
-        <v>197.5</v>
+        <v>19750</v>
       </c>
       <c r="I271" t="n">
-        <v>395.6000061035156</v>
+        <v>39560</v>
       </c>
       <c r="J271" t="n">
-        <v>1.003038005587421</v>
+        <v>1.003037974683544</v>
       </c>
       <c r="K271" s="1" t="n">
         <v>46100.625</v>
@@ -9137,10 +9137,10 @@
       </c>
       <c r="G272" t="inlineStr"/>
       <c r="H272" t="n">
-        <v>205</v>
+        <v>20500</v>
       </c>
       <c r="I272" t="n">
-        <v>205</v>
+        <v>20500</v>
       </c>
       <c r="J272" t="inlineStr"/>
       <c r="K272" s="1" t="n">
@@ -9167,13 +9167,13 @@
         <v>1</v>
       </c>
       <c r="G273" t="n">
-        <v>199.5</v>
+        <v>19950</v>
       </c>
       <c r="H273" t="n">
-        <v>205</v>
+        <v>20500</v>
       </c>
       <c r="I273" t="n">
-        <v>404.5</v>
+        <v>40450</v>
       </c>
       <c r="J273" t="n">
         <v>0.973170731707317</v>
@@ -9201,10 +9201,10 @@
       </c>
       <c r="G274" t="inlineStr"/>
       <c r="H274" t="n">
-        <v>210.1999969482422</v>
+        <v>21020</v>
       </c>
       <c r="I274" t="n">
-        <v>210.1999969482422</v>
+        <v>21020</v>
       </c>
       <c r="J274" t="inlineStr"/>
       <c r="K274" s="1" t="n">
@@ -9231,16 +9231,16 @@
         <v>1</v>
       </c>
       <c r="G275" t="n">
-        <v>199.5</v>
+        <v>19950</v>
       </c>
       <c r="H275" t="n">
-        <v>210.1999969482422</v>
+        <v>21020</v>
       </c>
       <c r="I275" t="n">
-        <v>409.6999969482422</v>
+        <v>40970</v>
       </c>
       <c r="J275" t="n">
-        <v>0.9490961127326902</v>
+        <v>0.9490960989533778</v>
       </c>
       <c r="K275" s="1" t="n">
         <v>46100.625</v>
@@ -9265,10 +9265,10 @@
       </c>
       <c r="G276" t="inlineStr"/>
       <c r="H276" t="n">
-        <v>213.1000061035156</v>
+        <v>21310</v>
       </c>
       <c r="I276" t="n">
-        <v>213.1000061035156</v>
+        <v>21310</v>
       </c>
       <c r="J276" t="inlineStr"/>
       <c r="K276" s="1" t="n">
@@ -9295,16 +9295,16 @@
         <v>1</v>
       </c>
       <c r="G277" t="n">
-        <v>197.6999969482422</v>
+        <v>19770</v>
       </c>
       <c r="H277" t="n">
-        <v>213.1000061035156</v>
+        <v>21310</v>
       </c>
       <c r="I277" t="n">
-        <v>410.8000030517578</v>
+        <v>41080</v>
       </c>
       <c r="J277" t="n">
-        <v>0.9277334175776949</v>
+        <v>0.9277334584702018</v>
       </c>
       <c r="K277" s="1" t="n">
         <v>46100.625</v>
@@ -9329,10 +9329,10 @@
       </c>
       <c r="G278" t="inlineStr"/>
       <c r="H278" t="n">
-        <v>208.5</v>
+        <v>20850</v>
       </c>
       <c r="I278" t="n">
-        <v>208.5</v>
+        <v>20850</v>
       </c>
       <c r="J278" t="inlineStr"/>
       <c r="K278" s="1" t="n">
@@ -9359,16 +9359,16 @@
         <v>1</v>
       </c>
       <c r="G279" t="n">
-        <v>193.1999969482422</v>
+        <v>19320</v>
       </c>
       <c r="H279" t="n">
-        <v>208.5</v>
+        <v>20850</v>
       </c>
       <c r="I279" t="n">
-        <v>401.6999969482422</v>
+        <v>40170</v>
       </c>
       <c r="J279" t="n">
-        <v>0.9266186903992431</v>
+        <v>0.9266187050359712</v>
       </c>
       <c r="K279" s="1" t="n">
         <v>46100.625</v>
@@ -9393,10 +9393,10 @@
       </c>
       <c r="G280" t="inlineStr"/>
       <c r="H280" t="n">
-        <v>198.6000061035156</v>
+        <v>19860</v>
       </c>
       <c r="I280" t="n">
-        <v>198.6000061035156</v>
+        <v>19860</v>
       </c>
       <c r="J280" t="inlineStr"/>
       <c r="K280" s="1" t="n">
@@ -9423,16 +9423,16 @@
         <v>1</v>
       </c>
       <c r="G281" t="n">
-        <v>195</v>
+        <v>19500</v>
       </c>
       <c r="H281" t="n">
-        <v>198.6000061035156</v>
+        <v>19860</v>
       </c>
       <c r="I281" t="n">
-        <v>393.6000061035156</v>
+        <v>39360</v>
       </c>
       <c r="J281" t="n">
-        <v>0.9818730816068595</v>
+        <v>0.9818731117824774</v>
       </c>
       <c r="K281" s="1" t="n">
         <v>46100.625</v>
@@ -9457,10 +9457,10 @@
       </c>
       <c r="G282" t="inlineStr"/>
       <c r="H282" t="n">
-        <v>197.6999969482422</v>
+        <v>19770</v>
       </c>
       <c r="I282" t="n">
-        <v>197.6999969482422</v>
+        <v>19770</v>
       </c>
       <c r="J282" t="inlineStr"/>
       <c r="K282" s="1" t="n">
@@ -9487,16 +9487,16 @@
         <v>1</v>
       </c>
       <c r="G283" t="n">
-        <v>200.8000030517578</v>
+        <v>20080</v>
       </c>
       <c r="H283" t="n">
-        <v>197.6999969482422</v>
+        <v>19770</v>
       </c>
       <c r="I283" t="n">
-        <v>398.5</v>
+        <v>39850</v>
       </c>
       <c r="J283" t="n">
-        <v>1.015680354837472</v>
+        <v>1.015680323722812</v>
       </c>
       <c r="K283" s="1" t="n">
         <v>46100.625</v>
@@ -9521,10 +9521,10 @@
       </c>
       <c r="G284" t="inlineStr"/>
       <c r="H284" t="n">
-        <v>198.1000061035156</v>
+        <v>19810</v>
       </c>
       <c r="I284" t="n">
-        <v>198.1000061035156</v>
+        <v>19810</v>
       </c>
       <c r="J284" t="inlineStr"/>
       <c r="K284" s="1" t="n">
@@ -9551,16 +9551,16 @@
         <v>1</v>
       </c>
       <c r="G285" t="n">
-        <v>205</v>
+        <v>20500</v>
       </c>
       <c r="H285" t="n">
-        <v>198.1000061035156</v>
+        <v>19810</v>
       </c>
       <c r="I285" t="n">
-        <v>403.1000061035156</v>
+        <v>40310</v>
       </c>
       <c r="J285" t="n">
-        <v>1.034830861604713</v>
+        <v>1.034830893488137</v>
       </c>
       <c r="K285" s="1" t="n">
         <v>46100.625</v>
@@ -9585,10 +9585,10 @@
       </c>
       <c r="G286" t="inlineStr"/>
       <c r="H286" t="n">
-        <v>189.5</v>
+        <v>18950</v>
       </c>
       <c r="I286" t="n">
-        <v>189.5</v>
+        <v>18950</v>
       </c>
       <c r="J286" t="inlineStr"/>
       <c r="K286" s="1" t="n">
@@ -9615,13 +9615,13 @@
         <v>1</v>
       </c>
       <c r="G287" t="n">
-        <v>211.5</v>
+        <v>21150</v>
       </c>
       <c r="H287" t="n">
-        <v>189.5</v>
+        <v>18950</v>
       </c>
       <c r="I287" t="n">
-        <v>401</v>
+        <v>40100</v>
       </c>
       <c r="J287" t="n">
         <v>1.116094986807388</v>
@@ -9649,10 +9649,10 @@
       </c>
       <c r="G288" t="inlineStr"/>
       <c r="H288" t="n">
-        <v>176.8999938964844</v>
+        <v>17690</v>
       </c>
       <c r="I288" t="n">
-        <v>176.8999938964844</v>
+        <v>17690</v>
       </c>
       <c r="J288" t="inlineStr"/>
       <c r="K288" s="1" t="n">
@@ -9679,16 +9679,16 @@
         <v>1</v>
       </c>
       <c r="G289" t="n">
-        <v>213.5</v>
+        <v>21350</v>
       </c>
       <c r="H289" t="n">
-        <v>176.8999938964844</v>
+        <v>17690</v>
       </c>
       <c r="I289" t="n">
-        <v>390.3999938964844</v>
+        <v>39040</v>
       </c>
       <c r="J289" t="n">
-        <v>1.206896593365247</v>
+        <v>1.206896551724138</v>
       </c>
       <c r="K289" s="1" t="n">
         <v>46100.625</v>
@@ -9713,10 +9713,10 @@
       </c>
       <c r="G290" t="inlineStr"/>
       <c r="H290" t="n">
-        <v>167.6999969482422</v>
+        <v>16770</v>
       </c>
       <c r="I290" t="n">
-        <v>167.6999969482422</v>
+        <v>16770</v>
       </c>
       <c r="J290" t="inlineStr"/>
       <c r="K290" s="1" t="n">
@@ -9743,16 +9743,16 @@
         <v>1</v>
       </c>
       <c r="G291" t="n">
-        <v>205</v>
+        <v>20500</v>
       </c>
       <c r="H291" t="n">
-        <v>167.6999969482422</v>
+        <v>16770</v>
       </c>
       <c r="I291" t="n">
-        <v>372.6999969482422</v>
+        <v>37270</v>
       </c>
       <c r="J291" t="n">
-        <v>1.222421012108127</v>
+        <v>1.22242098986285</v>
       </c>
       <c r="K291" s="1" t="n">
         <v>46100.625</v>
@@ -9816,7 +9816,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>100000.00</t>
+          <t>1000000.00</t>
         </is>
       </c>
     </row>
@@ -9828,7 +9828,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2052.60</t>
+          <t>205260.00</t>
         </is>
       </c>
     </row>
@@ -9946,7 +9946,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2052.60</t>
+          <t>205260.00</t>
         </is>
       </c>
     </row>
@@ -9958,7 +9958,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2098.60</t>
+          <t>209860.00</t>
         </is>
       </c>
     </row>
@@ -9970,7 +9970,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>4151.20</t>
+          <t>415120.00</t>
         </is>
       </c>
     </row>
@@ -9994,7 +9994,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>35411.70</t>
+          <t>3541170.00</t>
         </is>
       </c>
     </row>
@@ -10006,7 +10006,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>65713.10</t>
+          <t>6571310.00</t>
         </is>
       </c>
     </row>
@@ -10078,7 +10078,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>4151.20</t>
+          <t>415120.00</t>
         </is>
       </c>
     </row>
@@ -10102,7 +10102,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>4151.20</t>
+          <t>415120.00</t>
         </is>
       </c>
     </row>

</xml_diff>